<commit_message>
Update extract_final_cols and regenerate spreadsheet migration outputs
</commit_message>
<xml_diff>
--- a/S62aMigration/outputs/S62A_All_Sheets_migrated.xlsx
+++ b/S62aMigration/outputs/S62A_All_Sheets_migrated.xlsx
@@ -2326,7 +2326,11 @@
       <c r="BU3" s="11" t="n"/>
       <c r="BV3" s="14" t="n"/>
       <c r="BW3" s="11" t="n"/>
-      <c r="BX3" s="11" t="n"/>
+      <c r="BX3" s="57" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="BY3" s="12" t="n"/>
       <c r="BZ3" s="11" t="n"/>
       <c r="CA3" s="12" t="n"/>
@@ -2409,11 +2413,7 @@
       <c r="EH3" s="12" t="n"/>
       <c r="EI3" s="12" t="n"/>
       <c r="EJ3" s="12" t="n"/>
-      <c r="EK3" s="57" t="inlineStr">
-        <is>
-          <t>screening request received 7/4/22.  Negative screening direction issued 26/4/22</t>
-        </is>
-      </c>
+      <c r="EK3" s="11" t="n"/>
       <c r="EL3" s="12" t="n"/>
       <c r="EM3" s="12" t="n"/>
       <c r="EN3" s="11" t="n"/>
@@ -2464,7 +2464,11 @@
       <c r="GG3" s="11" t="n"/>
       <c r="GH3" s="11" t="n"/>
       <c r="GI3" s="11" t="n"/>
-      <c r="GJ3" s="11" t="n"/>
+      <c r="GJ3" s="57" t="inlineStr">
+        <is>
+          <t>screening request received 7/4/22.  Negative screening direction issued 26/4/22</t>
+        </is>
+      </c>
       <c r="GK3" s="11" t="n"/>
       <c r="GL3" s="11" t="n"/>
       <c r="GM3" s="11" t="n"/>
@@ -2476,7 +2480,11 @@
           <t>S62A/2022/0013</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="7" t="n"/>
       <c r="E4" s="59" t="inlineStr">
@@ -2602,11 +2610,7 @@
         </is>
       </c>
       <c r="CE4" s="7" t="n"/>
-      <c r="CF4" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF4" s="7" t="n"/>
       <c r="CG4" s="7" t="n"/>
       <c r="CH4" s="59" t="inlineStr">
         <is>
@@ -2709,11 +2713,7 @@
       <c r="EH4" s="20" t="n"/>
       <c r="EI4" s="20" t="n"/>
       <c r="EJ4" s="20" t="n"/>
-      <c r="EK4" s="59" t="inlineStr">
-        <is>
-          <t>Follow up from applicant asking for clarification - 31/1/23</t>
-        </is>
-      </c>
+      <c r="EK4" s="7" t="n"/>
       <c r="EL4" s="7" t="n"/>
       <c r="EM4" s="7" t="n"/>
       <c r="EN4" s="7" t="n"/>
@@ -2768,7 +2768,11 @@
       </c>
       <c r="GH4" s="7" t="n"/>
       <c r="GI4" s="7" t="n"/>
-      <c r="GJ4" s="7" t="n"/>
+      <c r="GJ4" s="59" t="inlineStr">
+        <is>
+          <t>Follow up from applicant asking for clarification - 31/1/23</t>
+        </is>
+      </c>
       <c r="GK4" s="7" t="n"/>
       <c r="GL4" s="7" t="n"/>
       <c r="GM4" s="7" t="n"/>
@@ -2780,7 +2784,11 @@
           <t>S62A/2022/0010</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
+      <c r="B5" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="59" t="inlineStr">
@@ -2902,7 +2910,7 @@
       <c r="BW5" s="7" t="n"/>
       <c r="BX5" s="59" t="inlineStr">
         <is>
-          <t>Luke Simpson (initial charging schedule done with Gemma Pannell)</t>
+          <t>Luke Simpson</t>
         </is>
       </c>
       <c r="BY5" s="20" t="n"/>
@@ -2916,11 +2924,7 @@
         </is>
       </c>
       <c r="CE5" s="7" t="n"/>
-      <c r="CF5" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF5" s="7" t="n"/>
       <c r="CG5" s="7" t="n"/>
       <c r="CH5" s="59" t="inlineStr">
         <is>
@@ -3294,11 +3298,7 @@
       <c r="EH6" s="20" t="n"/>
       <c r="EI6" s="20" t="n"/>
       <c r="EJ6" s="20" t="n"/>
-      <c r="EK6" s="59" t="inlineStr">
-        <is>
-          <t>WITHDRAWN 14/7/23</t>
-        </is>
-      </c>
+      <c r="EK6" s="7" t="n"/>
       <c r="EL6" s="7" t="n"/>
       <c r="EM6" s="7" t="n"/>
       <c r="EN6" s="7" t="n"/>
@@ -3349,7 +3349,11 @@
       <c r="GG6" s="7" t="n"/>
       <c r="GH6" s="7" t="n"/>
       <c r="GI6" s="7" t="n"/>
-      <c r="GJ6" s="7" t="n"/>
+      <c r="GJ6" s="59" t="inlineStr">
+        <is>
+          <t>WITHDRAWN 14/7/23</t>
+        </is>
+      </c>
       <c r="GK6" s="7" t="n"/>
       <c r="GL6" s="7" t="n"/>
       <c r="GM6" s="7" t="n"/>
@@ -3899,7 +3903,11 @@
           <t>S62A/2024/0033</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="59" t="inlineStr">
@@ -4303,11 +4311,7 @@
         </is>
       </c>
       <c r="CE10" s="7" t="n"/>
-      <c r="CF10" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF10" s="7" t="n"/>
       <c r="CG10" s="7" t="n"/>
       <c r="CH10" s="59" t="inlineStr">
         <is>
@@ -4410,11 +4414,7 @@
       <c r="EH10" s="20" t="n"/>
       <c r="EI10" s="20" t="n"/>
       <c r="EJ10" s="20" t="n"/>
-      <c r="EK10" s="59" t="inlineStr">
-        <is>
-          <t>Follow up advice issued to applicant (copied to LPA) on 20/5/24.  No charge for this.</t>
-        </is>
-      </c>
+      <c r="EK10" s="7" t="n"/>
       <c r="EL10" s="7" t="n"/>
       <c r="EM10" s="7" t="n"/>
       <c r="EN10" s="7" t="n"/>
@@ -4469,7 +4469,11 @@
       </c>
       <c r="GH10" s="7" t="n"/>
       <c r="GI10" s="7" t="n"/>
-      <c r="GJ10" s="7" t="n"/>
+      <c r="GJ10" s="59" t="inlineStr">
+        <is>
+          <t>Follow up advice issued to applicant (copied to LPA) on 20/5/24.  No charge for this.</t>
+        </is>
+      </c>
       <c r="GK10" s="7" t="n"/>
       <c r="GL10" s="7" t="n"/>
       <c r="GM10" s="7" t="n"/>
@@ -4481,7 +4485,11 @@
           <t>S62A/2024/0052</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="59" t="inlineStr">
@@ -4603,7 +4611,7 @@
       <c r="BW11" s="7" t="n"/>
       <c r="BX11" s="59" t="inlineStr">
         <is>
-          <t>Graham Chamberlain (available w/c 29 July).  Then on leave for 3 weeks from 9 Aug.</t>
+          <t>Graham Chamberlain</t>
         </is>
       </c>
       <c r="BY11" s="20" t="n"/>
@@ -4617,11 +4625,7 @@
         </is>
       </c>
       <c r="CE11" s="7" t="n"/>
-      <c r="CF11" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF11" s="7" t="n"/>
       <c r="CG11" s="7" t="n"/>
       <c r="CH11" s="59" t="inlineStr">
         <is>
@@ -4783,7 +4787,11 @@
           <t>S62A/2024/0074</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
+      <c r="B12" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="59" t="inlineStr">
@@ -5073,7 +5081,11 @@
           <t>S62A/2025/0086</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="59" t="inlineStr">
@@ -5368,7 +5380,11 @@
           <t>S62A/2025/0083</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
+      <c r="B14" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="59" t="inlineStr">
@@ -5648,7 +5664,11 @@
           <t>S62A/2022/0008</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B15" s="59" t="inlineStr">
+        <is>
+          <t>Closed - didn't proceed</t>
+        </is>
+      </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="59" t="inlineStr">
@@ -5868,11 +5888,7 @@
       <c r="EH15" s="20" t="n"/>
       <c r="EI15" s="20" t="n"/>
       <c r="EJ15" s="20" t="n"/>
-      <c r="EK15" s="59" t="inlineStr">
-        <is>
-          <t>Charging schedule shared with app 13/10/22.  Awaiting response.  App said they would request screening (from PINS?)  Told EST.  George prepared note with RP/PL re this possibly being an NSIP…</t>
-        </is>
-      </c>
+      <c r="EK15" s="7" t="n"/>
       <c r="EL15" s="7" t="n"/>
       <c r="EM15" s="7" t="n"/>
       <c r="EN15" s="7" t="n"/>
@@ -5923,7 +5939,11 @@
       <c r="GG15" s="7" t="n"/>
       <c r="GH15" s="7" t="n"/>
       <c r="GI15" s="7" t="n"/>
-      <c r="GJ15" s="7" t="n"/>
+      <c r="GJ15" s="59" t="inlineStr">
+        <is>
+          <t>Charging schedule shared with app 13/10/22.  Awaiting response.  App said they would request screening (from PINS?)  Told EST.  George prepared note with RP/PL re this possibly being an NSIP…</t>
+        </is>
+      </c>
       <c r="GK15" s="7" t="n"/>
       <c r="GL15" s="7" t="n"/>
       <c r="GM15" s="7" t="n"/>
@@ -5935,7 +5955,11 @@
           <t>S62A/2022/0009</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
+      <c r="B16" s="59" t="inlineStr">
+        <is>
+          <t>Closed - didn't proceed</t>
+        </is>
+      </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="59" t="inlineStr">
@@ -6438,11 +6462,7 @@
       <c r="EH17" s="20" t="n"/>
       <c r="EI17" s="20" t="n"/>
       <c r="EJ17" s="20" t="n"/>
-      <c r="EK17" s="59" t="inlineStr">
-        <is>
-          <t>Insp hours = 11.5</t>
-        </is>
-      </c>
+      <c r="EK17" s="7" t="n"/>
       <c r="EL17" s="7" t="n"/>
       <c r="EM17" s="7" t="n"/>
       <c r="EN17" s="7" t="n"/>
@@ -6497,7 +6517,11 @@
       </c>
       <c r="GH17" s="7" t="n"/>
       <c r="GI17" s="7" t="n"/>
-      <c r="GJ17" s="7" t="n"/>
+      <c r="GJ17" s="59" t="inlineStr">
+        <is>
+          <t>Insp hours = 11.5</t>
+        </is>
+      </c>
       <c r="GK17" s="7" t="n"/>
       <c r="GL17" s="7" t="n"/>
       <c r="GM17" s="7" t="n"/>
@@ -6509,7 +6533,11 @@
           <t>S62A/2025/0098</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="59" t="inlineStr">
@@ -6730,11 +6758,7 @@
       <c r="EH18" s="20" t="n"/>
       <c r="EI18" s="20" t="n"/>
       <c r="EJ18" s="20" t="n"/>
-      <c r="EK18" s="59" t="inlineStr">
-        <is>
-          <t>Insp hours = 16</t>
-        </is>
-      </c>
+      <c r="EK18" s="7" t="n"/>
       <c r="EL18" s="7" t="n"/>
       <c r="EM18" s="7" t="n"/>
       <c r="EN18" s="7" t="n"/>
@@ -6789,7 +6813,11 @@
       </c>
       <c r="GH18" s="7" t="n"/>
       <c r="GI18" s="7" t="n"/>
-      <c r="GJ18" s="7" t="n"/>
+      <c r="GJ18" s="59" t="inlineStr">
+        <is>
+          <t>Insp hours = 16</t>
+        </is>
+      </c>
       <c r="GK18" s="7" t="n"/>
       <c r="GL18" s="7" t="n"/>
       <c r="GM18" s="7" t="n"/>
@@ -6801,7 +6829,11 @@
           <t>S62A/2025/0100</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Closed - advice issued</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="59" t="inlineStr">
@@ -7016,11 +7048,7 @@
       <c r="EH19" s="20" t="n"/>
       <c r="EI19" s="20" t="n"/>
       <c r="EJ19" s="20" t="n"/>
-      <c r="EK19" s="59" t="inlineStr">
-        <is>
-          <t>Inspector hours 13.25</t>
-        </is>
-      </c>
+      <c r="EK19" s="7" t="n"/>
       <c r="EL19" s="7" t="n"/>
       <c r="EM19" s="7" t="n"/>
       <c r="EN19" s="7" t="n"/>
@@ -7075,7 +7103,11 @@
       </c>
       <c r="GH19" s="7" t="n"/>
       <c r="GI19" s="7" t="n"/>
-      <c r="GJ19" s="7" t="n"/>
+      <c r="GJ19" s="59" t="inlineStr">
+        <is>
+          <t>Inspector hours 13.25</t>
+        </is>
+      </c>
       <c r="GK19" s="7" t="n"/>
       <c r="GL19" s="7" t="n"/>
       <c r="GM19" s="7" t="n"/>
@@ -7407,9 +7439,7 @@
       <c r="AE21" s="60" t="n">
         <v>44763</v>
       </c>
-      <c r="AF21" s="60" t="n">
-        <v>44763</v>
-      </c>
+      <c r="AF21" s="20" t="n"/>
       <c r="AG21" s="60" t="n">
         <v>44755</v>
       </c>
@@ -7503,11 +7533,7 @@
         </is>
       </c>
       <c r="CE21" s="7" t="n"/>
-      <c r="CF21" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF21" s="7" t="n"/>
       <c r="CG21" s="7" t="n"/>
       <c r="CH21" s="59" t="inlineStr">
         <is>
@@ -7646,7 +7672,7 @@
       <c r="EJ21" s="20" t="n"/>
       <c r="EK21" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 5 Oct 2022; EIA Screening: 26/04/2022; 02/02/2022</t>
+          <t>EIA Screening: 26/04/2022; 02/02/2022</t>
         </is>
       </c>
       <c r="EL21" s="7" t="n"/>
@@ -7699,11 +7725,21 @@
           <t>payment details for MAG in pre-app folders</t>
         </is>
       </c>
-      <c r="GF21" s="7" t="n"/>
+      <c r="GF21" s="60" t="n">
+        <v>44895</v>
+      </c>
       <c r="GG21" s="7" t="n"/>
-      <c r="GH21" s="7" t="n"/>
-      <c r="GI21" s="7" t="n"/>
-      <c r="GJ21" s="7" t="n"/>
+      <c r="GH21" s="60" t="n">
+        <v>44718</v>
+      </c>
+      <c r="GI21" s="60" t="n">
+        <v>44705</v>
+      </c>
+      <c r="GJ21" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 5 Oct 2022</t>
+        </is>
+      </c>
       <c r="GK21" s="7" t="n"/>
       <c r="GL21" s="7" t="n"/>
       <c r="GM21" s="7" t="n"/>
@@ -7791,9 +7827,7 @@
       <c r="AD22" s="60" t="n">
         <v>44706</v>
       </c>
-      <c r="AE22" s="60" t="n">
-        <v>44764</v>
-      </c>
+      <c r="AE22" s="20" t="n"/>
       <c r="AF22" s="60" t="n">
         <v>44764</v>
       </c>
@@ -7896,11 +7930,7 @@
         </is>
       </c>
       <c r="CE22" s="7" t="n"/>
-      <c r="CF22" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF22" s="7" t="n"/>
       <c r="CG22" s="7" t="n"/>
       <c r="CH22" s="59" t="inlineStr">
         <is>
@@ -8030,7 +8060,7 @@
       <c r="EJ22" s="20" t="n"/>
       <c r="EK22" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 22 November 2022; EIA Screening: 28/04/2022; 13/05/2022</t>
+          <t>EIA Screening: 28/04/2022; 13/05/2022</t>
         </is>
       </c>
       <c r="EL22" s="7" t="n"/>
@@ -8083,11 +8113,21 @@
           <t>?</t>
         </is>
       </c>
-      <c r="GF22" s="7" t="n"/>
+      <c r="GF22" s="60" t="n">
+        <v>44854</v>
+      </c>
       <c r="GG22" s="7" t="n"/>
-      <c r="GH22" s="7" t="n"/>
-      <c r="GI22" s="7" t="n"/>
-      <c r="GJ22" s="7" t="n"/>
+      <c r="GH22" s="60" t="n">
+        <v>44677</v>
+      </c>
+      <c r="GI22" s="60" t="n">
+        <v>44665</v>
+      </c>
+      <c r="GJ22" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 22 November 2022</t>
+        </is>
+      </c>
       <c r="GK22" s="7" t="n"/>
       <c r="GL22" s="7" t="n"/>
       <c r="GM22" s="7" t="n"/>
@@ -8271,11 +8311,7 @@
         </is>
       </c>
       <c r="CE23" s="7" t="n"/>
-      <c r="CF23" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF23" s="7" t="n"/>
       <c r="CG23" s="7" t="n"/>
       <c r="CH23" s="59" t="inlineStr">
         <is>
@@ -8395,7 +8431,7 @@
       <c r="EJ23" s="20" t="n"/>
       <c r="EK23" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 23 May 2023; EIA Screening: 06/10/2022</t>
+          <t>EIA Screening: 06/10/2022</t>
         </is>
       </c>
       <c r="EL23" s="7" t="n"/>
@@ -8444,11 +8480,21 @@
       <c r="GC23" s="7" t="n"/>
       <c r="GD23" s="7" t="n"/>
       <c r="GE23" s="7" t="n"/>
-      <c r="GF23" s="7" t="n"/>
+      <c r="GF23" s="60" t="n">
+        <v>45030</v>
+      </c>
       <c r="GG23" s="7" t="n"/>
-      <c r="GH23" s="7" t="n"/>
-      <c r="GI23" s="7" t="n"/>
-      <c r="GJ23" s="7" t="n"/>
+      <c r="GH23" s="60" t="n">
+        <v>44852</v>
+      </c>
+      <c r="GI23" s="60" t="n">
+        <v>44846</v>
+      </c>
+      <c r="GJ23" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 23 May 2023</t>
+        </is>
+      </c>
       <c r="GK23" s="7" t="n"/>
       <c r="GL23" s="7" t="n"/>
       <c r="GM23" s="7" t="n"/>
@@ -8541,7 +8587,7 @@
         <v>44936</v>
       </c>
       <c r="AF24" s="60" t="n">
-        <v>44936</v>
+        <v>44972</v>
       </c>
       <c r="AG24" s="60" t="n">
         <v>44816</v>
@@ -8634,11 +8680,7 @@
         </is>
       </c>
       <c r="CE24" s="7" t="n"/>
-      <c r="CF24" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF24" s="7" t="n"/>
       <c r="CG24" s="7" t="n"/>
       <c r="CH24" s="59" t="inlineStr">
         <is>
@@ -8781,7 +8823,7 @@
       <c r="EJ24" s="20" t="n"/>
       <c r="EK24" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 20 June 2023.  PAP letter received 1/6/23.; EIA Screening: 20/07/2022; 19/08/2022</t>
+          <t>EIA Screening: 20/07/2022; 19/08/2022</t>
         </is>
       </c>
       <c r="EL24" s="7" t="n"/>
@@ -8830,11 +8872,21 @@
       <c r="GC24" s="7" t="n"/>
       <c r="GD24" s="7" t="n"/>
       <c r="GE24" s="7" t="n"/>
-      <c r="GF24" s="7" t="n"/>
+      <c r="GF24" s="60" t="n">
+        <v>45113</v>
+      </c>
       <c r="GG24" s="7" t="n"/>
-      <c r="GH24" s="7" t="n"/>
-      <c r="GI24" s="7" t="n"/>
-      <c r="GJ24" s="7" t="n"/>
+      <c r="GH24" s="60" t="n">
+        <v>44777</v>
+      </c>
+      <c r="GI24" s="60" t="n">
+        <v>44768</v>
+      </c>
+      <c r="GJ24" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 20 June 2023.  PAP letter received 1/6/23.</t>
+        </is>
+      </c>
       <c r="GK24" s="7" t="n"/>
       <c r="GL24" s="7" t="n"/>
       <c r="GM24" s="7" t="n"/>
@@ -9010,11 +9062,7 @@
         </is>
       </c>
       <c r="CE25" s="7" t="n"/>
-      <c r="CF25" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF25" s="7" t="n"/>
       <c r="CG25" s="7" t="n"/>
       <c r="CH25" s="59" t="inlineStr">
         <is>
@@ -9141,7 +9189,7 @@
       <c r="EJ25" s="20" t="n"/>
       <c r="EK25" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 22 June 2023; EIA Screening: 01/02/2023</t>
+          <t>EIA Screening: 01/02/2023</t>
         </is>
       </c>
       <c r="EL25" s="7" t="n"/>
@@ -9190,11 +9238,21 @@
       <c r="GC25" s="7" t="n"/>
       <c r="GD25" s="7" t="n"/>
       <c r="GE25" s="7" t="n"/>
-      <c r="GF25" s="7" t="n"/>
+      <c r="GF25" s="60" t="n">
+        <v>45148</v>
+      </c>
       <c r="GG25" s="7" t="n"/>
-      <c r="GH25" s="7" t="n"/>
-      <c r="GI25" s="7" t="n"/>
-      <c r="GJ25" s="7" t="n"/>
+      <c r="GH25" s="60" t="n">
+        <v>44973</v>
+      </c>
+      <c r="GI25" s="60" t="n">
+        <v>44964</v>
+      </c>
+      <c r="GJ25" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 22 June 2023</t>
+        </is>
+      </c>
       <c r="GK25" s="7" t="n"/>
       <c r="GL25" s="7" t="n"/>
       <c r="GM25" s="7" t="n"/>
@@ -9340,7 +9398,7 @@
       <c r="BW26" s="7" t="n"/>
       <c r="BX26" s="59" t="inlineStr">
         <is>
-          <t>Cullum Parker (prep day added for 17/8/22 for validation)</t>
+          <t>Cullum Parker</t>
         </is>
       </c>
       <c r="BY26" s="20" t="n"/>
@@ -9354,11 +9412,7 @@
         </is>
       </c>
       <c r="CE26" s="7" t="n"/>
-      <c r="CF26" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF26" s="7" t="n"/>
       <c r="CG26" s="7" t="n"/>
       <c r="CH26" s="59" t="inlineStr">
         <is>
@@ -9490,7 +9544,7 @@
       <c r="EJ26" s="20" t="n"/>
       <c r="EK26" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 22 June 2023; EIA Screening: 15/09/2022; 05/10/2022; 23/12/2022</t>
+          <t>EIA Screening: 15/09/2022; 05/10/2022; 23/12/2022</t>
         </is>
       </c>
       <c r="EL26" s="7" t="n"/>
@@ -9541,11 +9595,21 @@
       <c r="GE26" s="59" t="n">
         <v>125393</v>
       </c>
-      <c r="GF26" s="7" t="n"/>
+      <c r="GF26" s="60" t="n">
+        <v>45148</v>
+      </c>
       <c r="GG26" s="7" t="n"/>
-      <c r="GH26" s="7" t="n"/>
-      <c r="GI26" s="7" t="n"/>
-      <c r="GJ26" s="7" t="n"/>
+      <c r="GH26" s="60" t="n">
+        <v>44967</v>
+      </c>
+      <c r="GI26" s="60" t="n">
+        <v>44830</v>
+      </c>
+      <c r="GJ26" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 22 June 2023</t>
+        </is>
+      </c>
       <c r="GK26" s="7" t="n"/>
       <c r="GL26" s="7" t="n"/>
       <c r="GM26" s="7" t="n"/>
@@ -9633,7 +9697,7 @@
         <v>44943</v>
       </c>
       <c r="AE27" s="60" t="n">
-        <v>45007</v>
+        <v>44993</v>
       </c>
       <c r="AF27" s="60" t="n">
         <v>45007</v>
@@ -9729,11 +9793,7 @@
         </is>
       </c>
       <c r="CE27" s="7" t="n"/>
-      <c r="CF27" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF27" s="7" t="n"/>
       <c r="CG27" s="7" t="n"/>
       <c r="CH27" s="59" t="inlineStr">
         <is>
@@ -9848,7 +9908,7 @@
       <c r="EJ27" s="20" t="n"/>
       <c r="EK27" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 11 July 2023; EIA Screening: 30/11/2022</t>
+          <t>EIA Screening: 30/11/2022</t>
         </is>
       </c>
       <c r="EL27" s="7" t="n"/>
@@ -9899,9 +9959,17 @@
       <c r="GE27" s="7" t="n"/>
       <c r="GF27" s="7" t="n"/>
       <c r="GG27" s="7" t="n"/>
-      <c r="GH27" s="7" t="n"/>
-      <c r="GI27" s="7" t="n"/>
-      <c r="GJ27" s="7" t="n"/>
+      <c r="GH27" s="60" t="n">
+        <v>44903</v>
+      </c>
+      <c r="GI27" s="60" t="n">
+        <v>44900</v>
+      </c>
+      <c r="GJ27" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 11 July 2023</t>
+        </is>
+      </c>
       <c r="GK27" s="7" t="n"/>
       <c r="GL27" s="7" t="n"/>
       <c r="GM27" s="7" t="n"/>
@@ -9990,9 +10058,7 @@
       <c r="AD28" s="60" t="n">
         <v>44827</v>
       </c>
-      <c r="AE28" s="60" t="n">
-        <v>45002</v>
-      </c>
+      <c r="AE28" s="20" t="n"/>
       <c r="AF28" s="60" t="n">
         <v>45002</v>
       </c>
@@ -10095,11 +10161,7 @@
         </is>
       </c>
       <c r="CE28" s="7" t="n"/>
-      <c r="CF28" s="59" t="inlineStr">
-        <is>
-          <t>Helen Skinner/Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF28" s="7" t="n"/>
       <c r="CG28" s="7" t="n"/>
       <c r="CH28" s="59" t="inlineStr">
         <is>
@@ -10231,7 +10293,7 @@
       <c r="EJ28" s="20" t="n"/>
       <c r="EK28" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 26 July 2023; EIA Screening: 25/08/2022; 06/09/2022</t>
+          <t>EIA Screening: 25/08/2022; 06/09/2022</t>
         </is>
       </c>
       <c r="EL28" s="7" t="n"/>
@@ -10282,9 +10344,17 @@
       <c r="GE28" s="7" t="n"/>
       <c r="GF28" s="7" t="n"/>
       <c r="GG28" s="7" t="n"/>
-      <c r="GH28" s="7" t="n"/>
-      <c r="GI28" s="7" t="n"/>
-      <c r="GJ28" s="7" t="n"/>
+      <c r="GH28" s="60" t="n">
+        <v>44798</v>
+      </c>
+      <c r="GI28" s="60" t="n">
+        <v>44778</v>
+      </c>
+      <c r="GJ28" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 26 July 2023</t>
+        </is>
+      </c>
       <c r="GK28" s="7" t="n"/>
       <c r="GL28" s="7" t="n"/>
       <c r="GM28" s="7" t="n"/>
@@ -10468,11 +10538,7 @@
         </is>
       </c>
       <c r="CE29" s="7" t="n"/>
-      <c r="CF29" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF29" s="7" t="n"/>
       <c r="CG29" s="7" t="n"/>
       <c r="CH29" s="59" t="inlineStr">
         <is>
@@ -10593,7 +10659,7 @@
       <c r="EJ29" s="20" t="n"/>
       <c r="EK29" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 8 Aug 2023; EIA Screening: 01/11/2022</t>
+          <t>EIA Screening: 01/11/2022</t>
         </is>
       </c>
       <c r="EL29" s="7" t="n"/>
@@ -10644,9 +10710,17 @@
       <c r="GE29" s="7" t="n"/>
       <c r="GF29" s="7" t="n"/>
       <c r="GG29" s="7" t="n"/>
-      <c r="GH29" s="7" t="n"/>
-      <c r="GI29" s="7" t="n"/>
-      <c r="GJ29" s="7" t="n"/>
+      <c r="GH29" s="60" t="n">
+        <v>44873</v>
+      </c>
+      <c r="GI29" s="60" t="n">
+        <v>44757</v>
+      </c>
+      <c r="GJ29" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 8 Aug 2023</t>
+        </is>
+      </c>
       <c r="GK29" s="7" t="n"/>
       <c r="GL29" s="7" t="n"/>
       <c r="GM29" s="7" t="n"/>
@@ -10812,11 +10886,7 @@
         </is>
       </c>
       <c r="CE30" s="7" t="n"/>
-      <c r="CF30" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF30" s="7" t="n"/>
       <c r="CG30" s="7" t="n"/>
       <c r="CH30" s="59" t="inlineStr">
         <is>
@@ -10945,7 +11015,7 @@
       <c r="EJ30" s="20" t="n"/>
       <c r="EK30" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 7 Sept 2023; EIA Screening: 06/04/2023; 25/04/2023; 14/04/2023</t>
+          <t>EIA Screening: 06/04/2023; 25/04/2023; 14/04/2023</t>
         </is>
       </c>
       <c r="EL30" s="7" t="n"/>
@@ -10998,9 +11068,17 @@
       </c>
       <c r="GF30" s="7" t="n"/>
       <c r="GG30" s="7" t="n"/>
-      <c r="GH30" s="7" t="n"/>
-      <c r="GI30" s="7" t="n"/>
-      <c r="GJ30" s="7" t="n"/>
+      <c r="GH30" s="60" t="n">
+        <v>45040</v>
+      </c>
+      <c r="GI30" s="60" t="n">
+        <v>45033</v>
+      </c>
+      <c r="GJ30" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 7 Sept 2023</t>
+        </is>
+      </c>
       <c r="GK30" s="7" t="n"/>
       <c r="GL30" s="7" t="n"/>
       <c r="GM30" s="7" t="n"/>
@@ -11170,11 +11248,7 @@
         </is>
       </c>
       <c r="CE31" s="7" t="n"/>
-      <c r="CF31" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF31" s="7" t="n"/>
       <c r="CG31" s="7" t="n"/>
       <c r="CH31" s="59" t="inlineStr">
         <is>
@@ -11307,7 +11381,7 @@
       <c r="EJ31" s="20" t="n"/>
       <c r="EK31" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 20 Sept 2023; EIA Screening: 05/04/2023; 27/04/2023</t>
+          <t>EIA Screening: 05/04/2023; 27/04/2023</t>
         </is>
       </c>
       <c r="EL31" s="7" t="n"/>
@@ -11358,9 +11432,17 @@
       <c r="GE31" s="7" t="n"/>
       <c r="GF31" s="7" t="n"/>
       <c r="GG31" s="7" t="n"/>
-      <c r="GH31" s="7" t="n"/>
-      <c r="GI31" s="7" t="n"/>
-      <c r="GJ31" s="7" t="n"/>
+      <c r="GH31" s="60" t="n">
+        <v>45043</v>
+      </c>
+      <c r="GI31" s="60" t="n">
+        <v>45033</v>
+      </c>
+      <c r="GJ31" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 20 Sept 2023</t>
+        </is>
+      </c>
       <c r="GK31" s="7" t="n"/>
       <c r="GL31" s="7" t="n"/>
       <c r="GM31" s="7" t="n"/>
@@ -11534,11 +11616,7 @@
         </is>
       </c>
       <c r="CE32" s="7" t="n"/>
-      <c r="CF32" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF32" s="7" t="n"/>
       <c r="CG32" s="7" t="n"/>
       <c r="CH32" s="59" t="inlineStr">
         <is>
@@ -11672,7 +11750,7 @@
       <c r="EJ32" s="20" t="n"/>
       <c r="EK32" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 20 October 2023; EIA Screening: 11/04/2023</t>
+          <t>EIA Screening: 11/04/2023</t>
         </is>
       </c>
       <c r="EL32" s="7" t="n"/>
@@ -11723,11 +11801,21 @@
       <c r="GE32" s="59" t="n">
         <v>4620</v>
       </c>
-      <c r="GF32" s="7" t="n"/>
+      <c r="GF32" s="60" t="n">
+        <v>45219</v>
+      </c>
       <c r="GG32" s="7" t="n"/>
-      <c r="GH32" s="7" t="n"/>
-      <c r="GI32" s="7" t="n"/>
-      <c r="GJ32" s="7" t="n"/>
+      <c r="GH32" s="60" t="n">
+        <v>45043</v>
+      </c>
+      <c r="GI32" s="60" t="n">
+        <v>45036</v>
+      </c>
+      <c r="GJ32" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 20 October 2023</t>
+        </is>
+      </c>
       <c r="GK32" s="7" t="n"/>
       <c r="GL32" s="7" t="n"/>
       <c r="GM32" s="7" t="n"/>
@@ -11895,11 +11983,7 @@
         </is>
       </c>
       <c r="CE33" s="7" t="n"/>
-      <c r="CF33" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF33" s="7" t="n"/>
       <c r="CG33" s="7" t="n"/>
       <c r="CH33" s="59" t="inlineStr">
         <is>
@@ -12026,7 +12110,7 @@
       <c r="EJ33" s="20" t="n"/>
       <c r="EK33" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 12 December 2023; EIA Screening: 31/07/2023; 08/08/2023</t>
+          <t>EIA Screening: 31/07/2023; 08/08/2023</t>
         </is>
       </c>
       <c r="EL33" s="7" t="n"/>
@@ -12077,9 +12161,17 @@
       <c r="GE33" s="7" t="n"/>
       <c r="GF33" s="7" t="n"/>
       <c r="GG33" s="7" t="n"/>
-      <c r="GH33" s="7" t="n"/>
-      <c r="GI33" s="7" t="n"/>
-      <c r="GJ33" s="7" t="n"/>
+      <c r="GH33" s="60" t="n">
+        <v>45146</v>
+      </c>
+      <c r="GI33" s="60" t="n">
+        <v>45139</v>
+      </c>
+      <c r="GJ33" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 12 December 2023</t>
+        </is>
+      </c>
       <c r="GK33" s="7" t="n"/>
       <c r="GL33" s="7" t="n"/>
       <c r="GM33" s="7" t="n"/>
@@ -12166,9 +12258,7 @@
       <c r="AD34" s="60" t="n">
         <v>45176</v>
       </c>
-      <c r="AE34" s="60" t="n">
-        <v>45236</v>
-      </c>
+      <c r="AE34" s="20" t="n"/>
       <c r="AF34" s="60" t="n">
         <v>45236</v>
       </c>
@@ -12249,11 +12339,7 @@
         </is>
       </c>
       <c r="CE34" s="7" t="n"/>
-      <c r="CF34" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF34" s="7" t="n"/>
       <c r="CG34" s="7" t="n"/>
       <c r="CH34" s="59" t="inlineStr">
         <is>
@@ -12382,7 +12468,7 @@
       <c r="EJ34" s="20" t="n"/>
       <c r="EK34" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 26 Jan 2024.  HC challenge- Substantive hearing  11-12th June 2024 - 1.5 days.; EIA Screening: 21/06/2023; 03/08/2023</t>
+          <t>EIA Screening: 21/06/2023; 03/08/2023</t>
         </is>
       </c>
       <c r="EL34" s="7" t="n"/>
@@ -12435,9 +12521,17 @@
       </c>
       <c r="GF34" s="7" t="n"/>
       <c r="GG34" s="7" t="n"/>
-      <c r="GH34" s="7" t="n"/>
-      <c r="GI34" s="7" t="n"/>
-      <c r="GJ34" s="7" t="n"/>
+      <c r="GH34" s="60" t="n">
+        <v>45141</v>
+      </c>
+      <c r="GI34" s="60" t="n">
+        <v>45103</v>
+      </c>
+      <c r="GJ34" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 26 Jan 2024.  HC challenge- Substantive hearing  11-12th June 2024 - 1.5 days.</t>
+        </is>
+      </c>
       <c r="GK34" s="7" t="n"/>
       <c r="GL34" s="7" t="n"/>
       <c r="GM34" s="7" t="n"/>
@@ -12581,11 +12675,7 @@
         </is>
       </c>
       <c r="CE35" s="7" t="n"/>
-      <c r="CF35" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF35" s="7" t="n"/>
       <c r="CG35" s="7" t="n"/>
       <c r="CH35" s="59" t="inlineStr">
         <is>
@@ -12682,7 +12772,7 @@
       <c r="EJ35" s="20" t="n"/>
       <c r="EK35" s="59" t="inlineStr">
         <is>
-          <t>Withdrawn 22/12/23; EIA Screening: 06/12/2023</t>
+          <t>EIA Screening: 06/12/2023</t>
         </is>
       </c>
       <c r="EL35" s="7" t="n"/>
@@ -12735,7 +12825,11 @@
       <c r="GG35" s="7" t="n"/>
       <c r="GH35" s="7" t="n"/>
       <c r="GI35" s="7" t="n"/>
-      <c r="GJ35" s="7" t="n"/>
+      <c r="GJ35" s="59" t="inlineStr">
+        <is>
+          <t>Withdrawn 22/12/23</t>
+        </is>
+      </c>
       <c r="GK35" s="7" t="n"/>
       <c r="GL35" s="7" t="n"/>
       <c r="GM35" s="7" t="n"/>
@@ -12922,11 +13016,7 @@
         </is>
       </c>
       <c r="CE36" s="7" t="n"/>
-      <c r="CF36" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF36" s="7" t="n"/>
       <c r="CG36" s="7" t="n"/>
       <c r="CH36" s="59" t="inlineStr">
         <is>
@@ -13047,7 +13137,7 @@
       <c r="EJ36" s="20" t="n"/>
       <c r="EK36" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 8 April  2024; EIA Screening: 16/10/2023; 05/12/2023</t>
+          <t>EIA Screening: 16/10/2023; 05/12/2023</t>
         </is>
       </c>
       <c r="EL36" s="7" t="n"/>
@@ -13098,9 +13188,17 @@
       <c r="GE36" s="7" t="n"/>
       <c r="GF36" s="7" t="n"/>
       <c r="GG36" s="7" t="n"/>
-      <c r="GH36" s="7" t="n"/>
-      <c r="GI36" s="7" t="n"/>
-      <c r="GJ36" s="7" t="n"/>
+      <c r="GH36" s="60" t="n">
+        <v>45260</v>
+      </c>
+      <c r="GI36" s="60" t="n">
+        <v>45223</v>
+      </c>
+      <c r="GJ36" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 8 April  2024</t>
+        </is>
+      </c>
       <c r="GK36" s="7" t="n"/>
       <c r="GL36" s="7" t="n"/>
       <c r="GM36" s="7" t="n"/>
@@ -13274,11 +13372,7 @@
         </is>
       </c>
       <c r="CE37" s="7" t="n"/>
-      <c r="CF37" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF37" s="7" t="n"/>
       <c r="CG37" s="7" t="n"/>
       <c r="CH37" s="59" t="inlineStr">
         <is>
@@ -13403,7 +13497,7 @@
       <c r="EJ37" s="20" t="n"/>
       <c r="EK37" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 11 April  2024.  appeal on same site - 3331461. Let Andy Lumber know when decision issued; EIA Screening: 16/10/2023; 13/11/2023</t>
+          <t>EIA Screening: 16/10/2023; 13/11/2023</t>
         </is>
       </c>
       <c r="EL37" s="7" t="n"/>
@@ -13454,9 +13548,17 @@
       <c r="GE37" s="7" t="n"/>
       <c r="GF37" s="7" t="n"/>
       <c r="GG37" s="7" t="n"/>
-      <c r="GH37" s="7" t="n"/>
-      <c r="GI37" s="7" t="n"/>
-      <c r="GJ37" s="7" t="n"/>
+      <c r="GH37" s="60" t="n">
+        <v>45239</v>
+      </c>
+      <c r="GI37" s="60" t="n">
+        <v>45223</v>
+      </c>
+      <c r="GJ37" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 11 April  2024.  appeal on same site - 3331461. Let Andy Lumber know when decision issued</t>
+        </is>
+      </c>
       <c r="GK37" s="7" t="n"/>
       <c r="GL37" s="7" t="n"/>
       <c r="GM37" s="7" t="n"/>
@@ -13496,10 +13598,8 @@
       <c r="K38" s="60" t="n">
         <v>45160</v>
       </c>
-      <c r="L38" s="59" t="inlineStr">
-        <is>
-          <t>24/08/2023 (combined with invalid letter)</t>
-        </is>
+      <c r="L38" s="60" t="n">
+        <v>45162</v>
       </c>
       <c r="M38" s="60" t="n">
         <v>45202</v>
@@ -13630,11 +13730,7 @@
         </is>
       </c>
       <c r="CE38" s="7" t="n"/>
-      <c r="CF38" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF38" s="7" t="n"/>
       <c r="CG38" s="7" t="n"/>
       <c r="CH38" s="59" t="inlineStr">
         <is>
@@ -13765,7 +13861,7 @@
       <c r="EJ38" s="20" t="n"/>
       <c r="EK38" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 15 April  2024; EIA Screening: 24/08/2023; 28/09/2023</t>
+          <t>EIA Screening: 24/08/2023; 28/09/2023</t>
         </is>
       </c>
       <c r="EL38" s="7" t="n"/>
@@ -13814,11 +13910,21 @@
       <c r="GC38" s="7" t="n"/>
       <c r="GD38" s="7" t="n"/>
       <c r="GE38" s="7" t="n"/>
-      <c r="GF38" s="7" t="n"/>
+      <c r="GF38" s="60" t="n">
+        <v>45394</v>
+      </c>
       <c r="GG38" s="7" t="n"/>
-      <c r="GH38" s="7" t="n"/>
-      <c r="GI38" s="7" t="n"/>
-      <c r="GJ38" s="7" t="n"/>
+      <c r="GH38" s="60" t="n">
+        <v>45217</v>
+      </c>
+      <c r="GI38" s="60" t="n">
+        <v>45201</v>
+      </c>
+      <c r="GJ38" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 15 April  2024</t>
+        </is>
+      </c>
       <c r="GK38" s="7" t="n"/>
       <c r="GL38" s="7" t="n"/>
       <c r="GM38" s="7" t="n"/>
@@ -13986,11 +14092,7 @@
         </is>
       </c>
       <c r="CE39" s="7" t="n"/>
-      <c r="CF39" s="59" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
+      <c r="CF39" s="7" t="n"/>
       <c r="CG39" s="7" t="n"/>
       <c r="CH39" s="59" t="inlineStr">
         <is>
@@ -14111,7 +14213,7 @@
       <c r="EJ39" s="20" t="n"/>
       <c r="EK39" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 16 April  2024; EIA Screening: 06/11/2023; 12/12/2023</t>
+          <t>EIA Screening: 06/11/2023; 12/12/2023</t>
         </is>
       </c>
       <c r="EL39" s="7" t="n"/>
@@ -14162,9 +14264,17 @@
       <c r="GE39" s="7" t="n"/>
       <c r="GF39" s="7" t="n"/>
       <c r="GG39" s="7" t="n"/>
-      <c r="GH39" s="7" t="n"/>
-      <c r="GI39" s="7" t="n"/>
-      <c r="GJ39" s="7" t="n"/>
+      <c r="GH39" s="60" t="n">
+        <v>45267</v>
+      </c>
+      <c r="GI39" s="60" t="n">
+        <v>45243</v>
+      </c>
+      <c r="GJ39" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 16 April  2024</t>
+        </is>
+      </c>
       <c r="GK39" s="7" t="n"/>
       <c r="GL39" s="7" t="n"/>
       <c r="GM39" s="7" t="n"/>
@@ -14332,11 +14442,7 @@
         </is>
       </c>
       <c r="CE40" s="7" t="n"/>
-      <c r="CF40" s="59" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
+      <c r="CF40" s="7" t="n"/>
       <c r="CG40" s="7" t="n"/>
       <c r="CH40" s="59" t="inlineStr">
         <is>
@@ -14449,7 +14555,7 @@
       <c r="EJ40" s="20" t="n"/>
       <c r="EK40" s="59" t="inlineStr">
         <is>
-          <t>6 week challenge period 24 April  2024; EIA Screening: 24/10/2023; 21/11/2023</t>
+          <t>EIA Screening: 24/10/2023; 21/11/2023</t>
         </is>
       </c>
       <c r="EL40" s="7" t="n"/>
@@ -14500,9 +14606,15 @@
       <c r="GE40" s="7" t="n"/>
       <c r="GF40" s="7" t="n"/>
       <c r="GG40" s="7" t="n"/>
-      <c r="GH40" s="7" t="n"/>
+      <c r="GH40" s="60" t="n">
+        <v>45233</v>
+      </c>
       <c r="GI40" s="7" t="n"/>
-      <c r="GJ40" s="7" t="n"/>
+      <c r="GJ40" s="59" t="inlineStr">
+        <is>
+          <t>6 week challenge period 24 April  2024</t>
+        </is>
+      </c>
       <c r="GK40" s="7" t="n"/>
       <c r="GL40" s="7" t="n"/>
       <c r="GM40" s="7" t="n"/>
@@ -14587,7 +14699,7 @@
         <v>45184</v>
       </c>
       <c r="AE41" s="63" t="n">
-        <v>45233</v>
+        <v>45212</v>
       </c>
       <c r="AF41" s="63" t="n">
         <v>45233</v>
@@ -14628,11 +14740,6 @@
           <t>Leanne Palmer</t>
         </is>
       </c>
-      <c r="CF41" s="62" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
       <c r="CH41" s="62" t="inlineStr">
         <is>
           <t>Moors Fields</t>
@@ -14723,11 +14830,22 @@
       </c>
       <c r="EK41" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge period 8 May 2024; EIA Screening: 18/07/2023; 16/08/2023</t>
+          <t>EIA Screening: 18/07/2023; 16/08/2023</t>
         </is>
       </c>
       <c r="GE41" s="62" t="n">
         <v>38039</v>
+      </c>
+      <c r="GH41" s="63" t="n">
+        <v>45153</v>
+      </c>
+      <c r="GI41" s="63" t="n">
+        <v>45128</v>
+      </c>
+      <c r="GJ41" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge period 8 May 2024</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -14785,7 +14903,7 @@
         <v>45323</v>
       </c>
       <c r="AC42" s="63" t="n">
-        <v>45332</v>
+        <v>45351</v>
       </c>
       <c r="AD42" s="63" t="n">
         <v>45331</v>
@@ -14793,9 +14911,6 @@
       <c r="AE42" s="63" t="n">
         <v>45352</v>
       </c>
-      <c r="AF42" s="63" t="n">
-        <v>45352</v>
-      </c>
       <c r="AG42" s="63" t="n">
         <v>45334</v>
       </c>
@@ -14837,11 +14952,6 @@
           <t>Leanne Palmer</t>
         </is>
       </c>
-      <c r="CF42" s="62" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
       <c r="CH42" s="62" t="inlineStr">
         <is>
           <t>Land North of Thaxted Road</t>
@@ -14914,11 +15024,22 @@
       </c>
       <c r="EK42" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge period 22 May 2024; EIA Screening: 06/12/2023</t>
+          <t>EIA Screening: 06/12/2023</t>
         </is>
       </c>
       <c r="GE42" s="62" t="n">
         <v>13916</v>
+      </c>
+      <c r="GH42" s="63" t="n">
+        <v>45293</v>
+      </c>
+      <c r="GI42" s="63" t="n">
+        <v>45280</v>
+      </c>
+      <c r="GJ42" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge period 22 May 2024</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -14997,7 +15118,7 @@
         <v>45387</v>
       </c>
       <c r="AE43" s="63" t="n">
-        <v>45412</v>
+        <v>45398</v>
       </c>
       <c r="AF43" s="63" t="n">
         <v>45412</v>
@@ -15038,11 +15159,6 @@
           <t>Leanne Palmer</t>
         </is>
       </c>
-      <c r="CF43" s="62" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
       <c r="CH43" s="62" t="inlineStr">
         <is>
           <t>Land To The West Of Mill Lane Hatfield Heath</t>
@@ -15127,11 +15243,22 @@
       </c>
       <c r="EK43" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge period 5 July 2024; EIA Screening: 17/01/2024; 21/02/2024</t>
+          <t>EIA Screening: 17/01/2024; 21/02/2024</t>
         </is>
       </c>
       <c r="GE43" s="62" t="n">
         <v>4624</v>
+      </c>
+      <c r="GH43" s="63" t="n">
+        <v>45342</v>
+      </c>
+      <c r="GI43" s="63" t="n">
+        <v>45310</v>
+      </c>
+      <c r="GJ43" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge period 5 July 2024</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -15247,11 +15374,6 @@
           <t>Leanne Palmer</t>
         </is>
       </c>
-      <c r="CF44" s="62" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
       <c r="CH44" s="62" t="inlineStr">
         <is>
           <t>Land to the west of Clatterbury Lane</t>
@@ -15333,11 +15455,22 @@
       </c>
       <c r="EK44" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge 19 July 2024; EIA Screening: 06/12/2023</t>
+          <t>EIA Screening: 06/12/2023</t>
         </is>
       </c>
       <c r="GE44" s="62" t="n">
         <v>6070</v>
+      </c>
+      <c r="GH44" s="63" t="n">
+        <v>45307</v>
+      </c>
+      <c r="GI44" s="63" t="n">
+        <v>45279</v>
+      </c>
+      <c r="GJ44" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge 19 July 2024</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -15361,10 +15494,8 @@
           <t>Full Planning Application</t>
         </is>
       </c>
-      <c r="L45" s="62" t="inlineStr">
-        <is>
-          <t>Letter to app inviting further comments 25/10/2023</t>
-        </is>
+      <c r="L45" s="63" t="n">
+        <v>45224</v>
       </c>
       <c r="N45" s="63" t="n">
         <v>45245</v>
@@ -15425,11 +15556,6 @@
         </is>
       </c>
       <c r="CD45" s="62" t="inlineStr">
-        <is>
-          <t>Leanne Palmer</t>
-        </is>
-      </c>
-      <c r="CF45" s="62" t="inlineStr">
         <is>
           <t>Leanne Palmer</t>
         </is>
@@ -15512,7 +15638,15 @@
       </c>
       <c r="EK45" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge period 29 August 2024; REDETERMINED: S62A/22/0006RD</t>
+          <t>REDETERMINED: S62A/22/0006RD</t>
+        </is>
+      </c>
+      <c r="GH45" s="63" t="n">
+        <v>45258</v>
+      </c>
+      <c r="GJ45" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge period 29 August 2024</t>
         </is>
       </c>
     </row>
@@ -15718,11 +15852,22 @@
       </c>
       <c r="EK46" s="62" t="inlineStr">
         <is>
-          <t>6 week challenge 25 October 2024; EIA Screening: 19/06/2024</t>
+          <t>EIA Screening: 19/06/2024</t>
         </is>
       </c>
       <c r="GE46" s="62" t="n">
         <v>84126</v>
+      </c>
+      <c r="GH46" s="63" t="n">
+        <v>45469</v>
+      </c>
+      <c r="GI46" s="63" t="n">
+        <v>45462</v>
+      </c>
+      <c r="GJ46" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge 25 October 2024</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -15827,11 +15972,6 @@
           <t>Mark Boulton</t>
         </is>
       </c>
-      <c r="CF47" s="62" t="inlineStr">
-        <is>
-          <t>Mark Boulton</t>
-        </is>
-      </c>
       <c r="CH47" s="62" t="inlineStr">
         <is>
           <t>Land west of Thaxted Road</t>
@@ -15904,11 +16044,19 @@
       </c>
       <c r="EK47" s="62" t="inlineStr">
         <is>
-          <t>Repeat application (save for conditions) of UTT/23/2962/DFO.  BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 29 October 2024; EIA Screening: 31/07/2024</t>
+          <t>EIA Screening: 31/07/2024</t>
         </is>
       </c>
       <c r="GE47" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH47" s="63" t="n">
+        <v>45503</v>
+      </c>
+      <c r="GJ47" s="62" t="inlineStr">
+        <is>
+          <t>Repeat application (save for conditions) of UTT/23/2962/DFO.  BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 29 October 2024</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -15984,7 +16132,7 @@
         <v>45555</v>
       </c>
       <c r="AE48" s="63" t="n">
-        <v>45575</v>
+        <v>45561</v>
       </c>
       <c r="AF48" s="63" t="n">
         <v>45575</v>
@@ -16014,7 +16162,7 @@
       </c>
       <c r="BX48" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen - let Insp see LP email from UDC 09/08</t>
+          <t>Zoe Raygen</t>
         </is>
       </c>
       <c r="CH48" s="62" t="inlineStr">
@@ -16104,7 +16252,15 @@
       </c>
       <c r="EK48" s="62" t="inlineStr">
         <is>
-          <t>NPPF comments provided with application. BNG - yes - condition needed if approved. 6 week challenge 13 December 2024; EIA Screening: 25/07/2024; 15/08/2024</t>
+          <t>EIA Screening: 25/07/2024; 15/08/2024</t>
+        </is>
+      </c>
+      <c r="GH48" s="63" t="n">
+        <v>45516</v>
+      </c>
+      <c r="GJ48" s="62" t="inlineStr">
+        <is>
+          <t>NPPF comments provided with application. BNG - yes - condition needed if approved. 6 week challenge 13 December 2024</t>
         </is>
       </c>
     </row>
@@ -16178,7 +16334,7 @@
         <v>45510</v>
       </c>
       <c r="AE49" s="63" t="n">
-        <v>45541</v>
+        <v>45526</v>
       </c>
       <c r="AF49" s="63" t="n">
         <v>45541</v>
@@ -16317,11 +16473,22 @@
       </c>
       <c r="EK49" s="62" t="inlineStr">
         <is>
-          <t>BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 8 January 2025; EIA Screening: 25/06/2024; 16/07/2024</t>
+          <t>EIA Screening: 25/06/2024; 16/07/2024</t>
         </is>
       </c>
       <c r="GE49" s="62" t="n">
         <v>31270</v>
+      </c>
+      <c r="GH49" s="63" t="n">
+        <v>45481</v>
+      </c>
+      <c r="GI49" s="63" t="n">
+        <v>45474</v>
+      </c>
+      <c r="GJ49" s="62" t="inlineStr">
+        <is>
+          <t>BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 8 January 2025</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -16394,7 +16561,7 @@
         <v>45583</v>
       </c>
       <c r="AE50" s="63" t="n">
-        <v>45608</v>
+        <v>45594</v>
       </c>
       <c r="AF50" s="63" t="n">
         <v>45608</v>
@@ -16538,7 +16705,15 @@
       </c>
       <c r="EK50" s="62" t="inlineStr">
         <is>
-          <t>BNG - yes. NPPF ref back sent 13/12/2024. 6 Week challenge 28 Feb 2025; EIA Screening: 01/08/2024</t>
+          <t>EIA Screening: 01/08/2024</t>
+        </is>
+      </c>
+      <c r="GH50" s="63" t="n">
+        <v>45538</v>
+      </c>
+      <c r="GJ50" s="62" t="inlineStr">
+        <is>
+          <t>BNG - yes. NPPF ref back sent 13/12/2024. 6 Week challenge 28 Feb 2025</t>
         </is>
       </c>
     </row>
@@ -16563,10 +16738,8 @@
           <t>Full planning application</t>
         </is>
       </c>
-      <c r="L51" s="62" t="inlineStr">
-        <is>
-          <t>Stage 1 letter sent 30/08/2024. Further lettter sent 25/09/2024 re more time for response</t>
-        </is>
+      <c r="L51" s="63" t="n">
+        <v>45560</v>
       </c>
       <c r="N51" s="63" t="n">
         <v>45555</v>
@@ -16719,7 +16892,18 @@
       </c>
       <c r="EK51" s="62" t="inlineStr">
         <is>
-          <t>App - NPPF comments invited 19/12; REDETERMINED: S62A/2023/0019RD; EIA Screening: 21/11/2024; 11/12/2024</t>
+          <t>REDETERMINED: S62A/2023/0019RD; EIA Screening: 21/11/2024; 11/12/2024</t>
+        </is>
+      </c>
+      <c r="GH51" s="63" t="n">
+        <v>45625</v>
+      </c>
+      <c r="GI51" s="63" t="n">
+        <v>45103</v>
+      </c>
+      <c r="GJ51" s="62" t="inlineStr">
+        <is>
+          <t>App - NPPF comments invited 19/12</t>
         </is>
       </c>
     </row>
@@ -16825,7 +17009,12 @@
       </c>
       <c r="EK52" s="62" t="inlineStr">
         <is>
-          <t>BNG condition applies.  Sent to Inspector for validation 9/4 ST; EIA Screening: 03/04/2025</t>
+          <t>EIA Screening: 03/04/2025</t>
+        </is>
+      </c>
+      <c r="GJ52" s="62" t="inlineStr">
+        <is>
+          <t>BNG condition applies.  Sent to Inspector for validation 9/4 ST</t>
         </is>
       </c>
     </row>
@@ -16905,7 +17094,7 @@
         <v>45730</v>
       </c>
       <c r="AE53" s="63" t="n">
-        <v>45763</v>
+        <v>45749</v>
       </c>
       <c r="AF53" s="63" t="n">
         <v>45763</v>
@@ -16946,7 +17135,7 @@
       </c>
       <c r="BX53" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validating</t>
+          <t>Zoe Raygen (v)</t>
         </is>
       </c>
       <c r="BZ53" s="62" t="inlineStr">
@@ -17033,11 +17222,19 @@
       </c>
       <c r="EK53" s="62" t="inlineStr">
         <is>
-          <t>BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 8 January 2025; EIA Screening: 15/01/2025</t>
+          <t>EIA Screening: 15/01/2025</t>
         </is>
       </c>
       <c r="GE53" s="62" t="n">
         <v>31790</v>
+      </c>
+      <c r="GH53" s="63" t="n">
+        <v>45684</v>
+      </c>
+      <c r="GJ53" s="62" t="inlineStr">
+        <is>
+          <t>BNG - reserved matters so not required BNG PPG 003.https://www.gov.uk/guidance/biodiversity-net-gain#about-biodiversity-gain. 6 week challenge 8 January 2025</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -17164,7 +17361,12 @@
       </c>
       <c r="BX54" s="62" t="inlineStr">
         <is>
-          <t>Cullum Parker validating. HG Insp needed Zoe Raygen</t>
+          <t>Cullum Parker (v)</t>
+        </is>
+      </c>
+      <c r="BZ54" s="62" t="inlineStr">
+        <is>
+          <t>Zoe Raygen</t>
         </is>
       </c>
       <c r="CH54" s="62" t="inlineStr">
@@ -17243,7 +17445,15 @@
       </c>
       <c r="EK54" s="62" t="inlineStr">
         <is>
-          <t>BNG condition applies; EIA Screening: 15/01/2025; 24/02/2025</t>
+          <t>EIA Screening: 15/01/2025; 24/02/2025</t>
+        </is>
+      </c>
+      <c r="GH54" s="63" t="n">
+        <v>45705</v>
+      </c>
+      <c r="GJ54" s="62" t="inlineStr">
+        <is>
+          <t>BNG condition applies</t>
         </is>
       </c>
     </row>
@@ -17349,11 +17559,8 @@
       </c>
       <c r="BX55" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validating</t>
-        </is>
-      </c>
-      <c r="BY55" s="63" t="n">
-        <v>45814</v>
+          <t>Zoe Raygen (v)</t>
+        </is>
       </c>
       <c r="BZ55" s="62" t="inlineStr">
         <is>
@@ -17445,7 +17652,15 @@
       </c>
       <c r="EK55" s="62" t="inlineStr">
         <is>
-          <t>BNG condition applies; EIA Screening: 13/05/2025</t>
+          <t>EIA Screening: 13/05/2025</t>
+        </is>
+      </c>
+      <c r="GH55" s="63" t="n">
+        <v>45807</v>
+      </c>
+      <c r="GJ55" s="62" t="inlineStr">
+        <is>
+          <t>BNG condition applies</t>
         </is>
       </c>
     </row>
@@ -17877,11 +18092,6 @@
           <t>B Thandi</t>
         </is>
       </c>
-      <c r="CE60" s="62" t="inlineStr">
-        <is>
-          <t>B Thandi</t>
-        </is>
-      </c>
       <c r="CG60" s="62" t="inlineStr">
         <is>
           <t>Mike Robins/David Morgan</t>
@@ -17954,13 +18164,16 @@
       <c r="EH60" s="63" t="n">
         <v>45441</v>
       </c>
-      <c r="EK60" s="62" t="inlineStr">
-        <is>
-          <t>CIL - make sure DL gets the correct wording. LPA say CIL liable but Nil return.  David Morgan to review re HG aspects. 6 Week challenge date 10 July 2024</t>
-        </is>
-      </c>
       <c r="GE60" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH60" s="63" t="n">
+        <v>45393</v>
+      </c>
+      <c r="GJ60" s="62" t="inlineStr">
+        <is>
+          <t>CIL - make sure DL gets the correct wording. LPA say CIL liable but Nil return.  David Morgan to review re HG aspects. 6 Week challenge date 10 July 2024</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -18076,11 +18289,6 @@
           <t>B Thandi</t>
         </is>
       </c>
-      <c r="CE61" s="62" t="inlineStr">
-        <is>
-          <t>B Thandi</t>
-        </is>
-      </c>
       <c r="CG61" s="62" t="inlineStr">
         <is>
           <t>Mike Robins</t>
@@ -18143,13 +18351,16 @@
       <c r="EH61" s="63" t="n">
         <v>45448</v>
       </c>
-      <c r="EK61" s="62" t="inlineStr">
-        <is>
-          <t>6 week challenge 17 July 2024</t>
-        </is>
-      </c>
       <c r="GE61" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH61" s="63" t="n">
+        <v>45392</v>
+      </c>
+      <c r="GJ61" s="62" t="inlineStr">
+        <is>
+          <t>6 week challenge 17 July 2024</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -18265,11 +18476,6 @@
           <t>Jonathan Edwards</t>
         </is>
       </c>
-      <c r="CE62" s="62" t="inlineStr">
-        <is>
-          <t>Jonathan Edwards</t>
-        </is>
-      </c>
       <c r="CG62" s="62" t="inlineStr">
         <is>
           <t>Zoe Raygen</t>
@@ -18332,13 +18538,19 @@
       <c r="EH62" s="63" t="n">
         <v>45464</v>
       </c>
-      <c r="EK62" s="62" t="inlineStr">
-        <is>
-          <t>BNG? 6 week challenge 2 August 2024</t>
-        </is>
-      </c>
       <c r="GE62" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH62" s="63" t="n">
+        <v>45419</v>
+      </c>
+      <c r="GI62" s="63" t="n">
+        <v>45413</v>
+      </c>
+      <c r="GJ62" s="62" t="inlineStr">
+        <is>
+          <t>BNG? 6 week challenge 2 August 2024</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -18458,11 +18670,6 @@
           <t>B Thandi</t>
         </is>
       </c>
-      <c r="CE63" s="62" t="inlineStr">
-        <is>
-          <t>B Thandi</t>
-        </is>
-      </c>
       <c r="CH63" s="62" t="inlineStr">
         <is>
           <t>85 Ruby Street</t>
@@ -18507,13 +18714,19 @@
       <c r="EA63" s="63" t="n">
         <v>45427</v>
       </c>
-      <c r="EK63" s="62" t="inlineStr">
-        <is>
-          <t>Declined jurisdiction as retrospective application.  Fee to be returned.</t>
-        </is>
-      </c>
       <c r="GE63" s="62" t="n">
         <v>568</v>
+      </c>
+      <c r="GH63" s="63" t="n">
+        <v>45428</v>
+      </c>
+      <c r="GI63" s="63" t="n">
+        <v>45427</v>
+      </c>
+      <c r="GJ63" s="62" t="inlineStr">
+        <is>
+          <t>Declined jurisdiction as retrospective application.  Fee to be returned.</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -18540,10 +18753,8 @@
       <c r="K64" s="63" t="n">
         <v>45365</v>
       </c>
-      <c r="L64" s="62" t="inlineStr">
-        <is>
-          <t>27/03/2024 - combined with letter 8</t>
-        </is>
+      <c r="L64" s="63" t="n">
+        <v>45378</v>
       </c>
       <c r="M64" s="63" t="n">
         <v>45378</v>
@@ -18589,9 +18800,6 @@
       <c r="AD64" s="63" t="n">
         <v>45469</v>
       </c>
-      <c r="AE64" s="63" t="n">
-        <v>45481</v>
-      </c>
       <c r="AF64" s="63" t="n">
         <v>45481</v>
       </c>
@@ -18652,11 +18860,6 @@
           <t>H Hockenhall</t>
         </is>
       </c>
-      <c r="CE64" s="62" t="inlineStr">
-        <is>
-          <t>H Hockenhall</t>
-        </is>
-      </c>
       <c r="CH64" s="62" t="inlineStr">
         <is>
           <t>57 Prince Street</t>
@@ -18713,13 +18916,16 @@
       <c r="EA64" s="63" t="n">
         <v>45432</v>
       </c>
-      <c r="EK64" s="62" t="inlineStr">
-        <is>
-          <t>Withdrawn 08/07/2024</t>
-        </is>
-      </c>
       <c r="GE64" s="62" t="n">
         <v>258</v>
+      </c>
+      <c r="GH64" s="63" t="n">
+        <v>45440</v>
+      </c>
+      <c r="GJ64" s="62" t="inlineStr">
+        <is>
+          <t>Withdrawn 08/07/2024</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -18832,11 +19038,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE65" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH65" s="62" t="inlineStr">
         <is>
           <t>9a / 9b Rosebery Avenue</t>
@@ -18897,13 +19098,19 @@
       <c r="EH65" s="63" t="n">
         <v>45519</v>
       </c>
-      <c r="EK65" s="62" t="inlineStr">
-        <is>
-          <t>App says BNG exempt. No need to ref back on NPPF / WMS.  6 week challenge 26 Sept.</t>
-        </is>
-      </c>
       <c r="GE65" s="62" t="n">
         <v>624</v>
+      </c>
+      <c r="GH65" s="63" t="n">
+        <v>45483</v>
+      </c>
+      <c r="GI65" s="63" t="n">
+        <v>45449</v>
+      </c>
+      <c r="GJ65" s="62" t="inlineStr">
+        <is>
+          <t>App says BNG exempt. No need to ref back on NPPF / WMS.  6 week challenge 26 Sept.</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -19020,11 +19227,6 @@
           <t>Darren Hendley</t>
         </is>
       </c>
-      <c r="CE66" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley</t>
-        </is>
-      </c>
       <c r="CH66" s="62" t="inlineStr">
         <is>
           <t>87 Queenshill Road</t>
@@ -19083,7 +19285,13 @@
       <c r="EH66" s="63" t="n">
         <v>45523</v>
       </c>
-      <c r="EK66" s="62" t="inlineStr">
+      <c r="GH66" s="63" t="n">
+        <v>45476</v>
+      </c>
+      <c r="GI66" s="63" t="n">
+        <v>45450</v>
+      </c>
+      <c r="GJ66" s="62" t="inlineStr">
         <is>
           <t>App says BNG exempt. NPPF ref back 31/07. Responses due 07/08. 6 Week challenge 30 Sept 2024</t>
         </is>
@@ -19191,11 +19399,6 @@
           <t>Jonathan Edwards</t>
         </is>
       </c>
-      <c r="CE67" s="62" t="inlineStr">
-        <is>
-          <t>Jonathan Edwards</t>
-        </is>
-      </c>
       <c r="CH67" s="62" t="inlineStr">
         <is>
           <t>59 Langton Road</t>
@@ -19256,13 +19459,22 @@
       <c r="EH67" s="63" t="n">
         <v>45526</v>
       </c>
-      <c r="EK67" s="62" t="inlineStr">
-        <is>
-          <t>App says BNG exempt.  De minimis. NPPF / WMS ref back 06/08/24. 6 week challenge 3 October 2024</t>
-        </is>
-      </c>
       <c r="GE67" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GF67" s="63" t="n">
+        <v>45587</v>
+      </c>
+      <c r="GH67" s="63" t="n">
+        <v>45476</v>
+      </c>
+      <c r="GI67" s="63" t="n">
+        <v>45469</v>
+      </c>
+      <c r="GJ67" s="62" t="inlineStr">
+        <is>
+          <t>App says BNG exempt.  De minimis. NPPF / WMS ref back 06/08/24. 6 week challenge 3 October 2024</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -19369,11 +19581,6 @@
           <t>Helen Hockenhull</t>
         </is>
       </c>
-      <c r="CE68" s="62" t="inlineStr">
-        <is>
-          <t>Rebecca Dickson (APO) / Helen Hockenhull</t>
-        </is>
-      </c>
       <c r="CH68" s="62" t="inlineStr">
         <is>
           <t>39-43 College Green</t>
@@ -19436,13 +19643,16 @@
       <c r="EH68" s="63" t="n">
         <v>45531</v>
       </c>
-      <c r="EK68" s="62" t="inlineStr">
-        <is>
-          <t>App says BNG exempt (no habitate on site) No NPPF ref back needed. 6 Week challenge 8 October 2024</t>
-        </is>
-      </c>
       <c r="GE68" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH68" s="63" t="n">
+        <v>45481</v>
+      </c>
+      <c r="GJ68" s="62" t="inlineStr">
+        <is>
+          <t>App says BNG exempt (no habitate on site) No NPPF ref back needed. 6 Week challenge 8 October 2024</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -19558,11 +19768,6 @@
           <t>Andreea Spataru (APO)</t>
         </is>
       </c>
-      <c r="CE69" s="62" t="inlineStr">
-        <is>
-          <t>Andreea Spataru (APO)/ and ???</t>
-        </is>
-      </c>
       <c r="CH69" s="62" t="inlineStr">
         <is>
           <t>Vintry House (sixth floor)</t>
@@ -19625,7 +19830,10 @@
       <c r="EH69" s="63" t="n">
         <v>45552</v>
       </c>
-      <c r="EK69" s="62" t="inlineStr">
+      <c r="GH69" s="63" t="n">
+        <v>45505</v>
+      </c>
+      <c r="GJ69" s="62" t="inlineStr">
         <is>
           <t>NPPF comments asked for. BNG exempt. 6 Week challenge 29 October 2024</t>
         </is>
@@ -19749,11 +19957,6 @@
           <t>Zoe Raygen</t>
         </is>
       </c>
-      <c r="CE70" s="62" t="inlineStr">
-        <is>
-          <t>Andreea Spataru (APO)/ and Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH70" s="62" t="inlineStr">
         <is>
           <t>1 Repton Road</t>
@@ -19813,7 +20016,10 @@
       <c r="EH70" s="63" t="n">
         <v>45553</v>
       </c>
-      <c r="EK70" s="62" t="inlineStr">
+      <c r="GH70" s="63" t="n">
+        <v>45506</v>
+      </c>
+      <c r="GJ70" s="62" t="inlineStr">
         <is>
           <t>NPPF comments asked for. BNG exempt. 6 Week challenge 30 October 2024</t>
         </is>
@@ -19943,11 +20149,6 @@
           <t>Hannah Ellison</t>
         </is>
       </c>
-      <c r="CE71" s="62" t="inlineStr">
-        <is>
-          <t>Hannah Ellison</t>
-        </is>
-      </c>
       <c r="CG71" s="62" t="inlineStr">
         <is>
           <t>Rebecca</t>
@@ -20020,13 +20221,16 @@
       <c r="EH71" s="63" t="n">
         <v>45559</v>
       </c>
-      <c r="EK71" s="62" t="inlineStr">
-        <is>
-          <t>No comments needed on NPPF / WMS. BNG condition applies if approved. 6 week 5 November 2024</t>
-        </is>
-      </c>
       <c r="GE71" s="62" t="n">
         <v>293</v>
+      </c>
+      <c r="GH71" s="63" t="n">
+        <v>45512</v>
+      </c>
+      <c r="GJ71" s="62" t="inlineStr">
+        <is>
+          <t>No comments needed on NPPF / WMS. BNG condition applies if approved. 6 week 5 November 2024</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -20110,7 +20314,7 @@
         </is>
       </c>
       <c r="AM72" s="64" t="n">
-        <v>40426.41666666666</v>
+        <v>46270.41666666666</v>
       </c>
       <c r="AS72" s="62" t="inlineStr">
         <is>
@@ -20139,12 +20343,7 @@
       </c>
       <c r="BX72" s="62" t="inlineStr">
         <is>
-          <t>Jennifer Wallace (was Downs)</t>
-        </is>
-      </c>
-      <c r="CE72" s="62" t="inlineStr">
-        <is>
-          <t>Jennifer Wallace (was Downs)</t>
+          <t>Jennifer Wallace</t>
         </is>
       </c>
       <c r="CG72" s="62" t="inlineStr">
@@ -20204,13 +20403,19 @@
       <c r="EH72" s="63" t="n">
         <v>45574</v>
       </c>
-      <c r="EK72" s="62" t="inlineStr">
-        <is>
-          <t>App says BNG exempt (self build). Comments on NPPF / WMS not needed as neutral in terms of housing numbers.</t>
-        </is>
-      </c>
       <c r="GE72" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH72" s="63" t="n">
+        <v>45517</v>
+      </c>
+      <c r="GI72" s="63" t="n">
+        <v>45463</v>
+      </c>
+      <c r="GJ72" s="62" t="inlineStr">
+        <is>
+          <t>App says BNG exempt (self build). Comments on NPPF / WMS not needed as neutral in terms of housing numbers.</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -20318,12 +20523,7 @@
       </c>
       <c r="BX73" s="62" t="inlineStr">
         <is>
-          <t>Jennifer Wallace (was Downs)</t>
-        </is>
-      </c>
-      <c r="CE73" s="62" t="inlineStr">
-        <is>
-          <t>Jennifer Wallace (was Downs)</t>
+          <t>Jennifer Wallace</t>
         </is>
       </c>
       <c r="CH73" s="62" t="inlineStr">
@@ -20375,7 +20575,10 @@
       <c r="EH73" s="63" t="n">
         <v>45587</v>
       </c>
-      <c r="EK73" s="62" t="inlineStr">
+      <c r="GH73" s="63" t="n">
+        <v>45540</v>
+      </c>
+      <c r="GJ73" s="62" t="inlineStr">
         <is>
           <t>App says BNG exempt (self build). No comments needed on NPPF / WMS. 6 week date 3 December 2024</t>
         </is>
@@ -20492,12 +20695,12 @@
       </c>
       <c r="BX74" s="62" t="inlineStr">
         <is>
-          <t>Jonathan Edwards (Zoe Raygen validating)</t>
-        </is>
-      </c>
-      <c r="CE74" s="62" t="inlineStr">
-        <is>
-          <t>Jonathan Edwards (Zoe Raygen validating)</t>
+          <t>Zoe Raygen (v)</t>
+        </is>
+      </c>
+      <c r="BZ74" s="62" t="inlineStr">
+        <is>
+          <t>Jonathan Edwards</t>
         </is>
       </c>
       <c r="CH74" s="62" t="inlineStr">
@@ -20567,7 +20770,10 @@
       <c r="EH74" s="63" t="n">
         <v>45589</v>
       </c>
-      <c r="EK74" s="62" t="inlineStr">
+      <c r="GH74" s="63" t="n">
+        <v>45546</v>
+      </c>
+      <c r="GJ74" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">BNG info not provided (exemption of below threshold claimed).  </t>
         </is>
@@ -20645,7 +20851,7 @@
           <t>principle of development, parking, neighbour amenity</t>
         </is>
       </c>
-      <c r="EK75" s="62" t="inlineStr">
+      <c r="GJ75" s="62" t="inlineStr">
         <is>
           <t>App said no longer being submitted under S62A.  21/10/24</t>
         </is>
@@ -20744,11 +20950,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE76" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH76" s="62" t="inlineStr">
         <is>
           <t>Unit H</t>
@@ -20818,7 +21019,10 @@
       <c r="EH76" s="63" t="n">
         <v>45611</v>
       </c>
-      <c r="EK76" s="62" t="inlineStr">
+      <c r="GH76" s="63" t="n">
+        <v>45572</v>
+      </c>
+      <c r="GJ76" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed.  De minimis. 6 week date 27 December 2024.</t>
         </is>
@@ -20925,11 +21129,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE77" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH77" s="62" t="inlineStr">
         <is>
           <t>59 Langton Road</t>
@@ -20989,7 +21188,10 @@
       <c r="EH77" s="63" t="n">
         <v>45614</v>
       </c>
-      <c r="EK77" s="62" t="inlineStr">
+      <c r="GH77" s="63" t="n">
+        <v>45565</v>
+      </c>
+      <c r="GJ77" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed.  De minimis. 6 week date 30 December 2024</t>
         </is>
@@ -21106,11 +21308,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE78" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH78" s="62" t="inlineStr">
         <is>
           <t>Cotham School</t>
@@ -21188,13 +21385,16 @@
       <c r="EH78" s="63" t="n">
         <v>45644</v>
       </c>
-      <c r="EK78" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed.  De minimis. NPPF ref back not needed. 6 week date 29 January 2025</t>
-        </is>
-      </c>
       <c r="GE78" s="62" t="n">
         <v>293</v>
+      </c>
+      <c r="GH78" s="63" t="n">
+        <v>45590</v>
+      </c>
+      <c r="GJ78" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed.  De minimis. NPPF ref back not needed. 6 week date 29 January 2025</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -21308,11 +21508,6 @@
           <t>Gareth Fort</t>
         </is>
       </c>
-      <c r="CE79" s="62" t="inlineStr">
-        <is>
-          <t>Gareth Fort</t>
-        </is>
-      </c>
       <c r="CH79" s="62" t="inlineStr">
         <is>
           <t>Redcliff Quay</t>
@@ -21390,7 +21585,10 @@
       <c r="EH79" s="63" t="n">
         <v>45646</v>
       </c>
-      <c r="EK79" s="62" t="inlineStr">
+      <c r="GH79" s="63" t="n">
+        <v>45597</v>
+      </c>
+      <c r="GJ79" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed.  De minimis. NPPF ref back not needed</t>
         </is>
@@ -21501,11 +21699,6 @@
           <t>Insp Zoe Raygen</t>
         </is>
       </c>
-      <c r="CE80" s="62" t="inlineStr">
-        <is>
-          <t>Rebecca Dickson (APO) / Insp Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH80" s="62" t="inlineStr">
         <is>
           <t>23 Hillsborough Road</t>
@@ -21565,13 +21758,16 @@
       <c r="EH80" s="63" t="n">
         <v>45667</v>
       </c>
-      <c r="EK80" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis. NPPF ref back comments from app requested 17/12</t>
-        </is>
-      </c>
       <c r="GE80" s="62" t="n">
         <v>293</v>
+      </c>
+      <c r="GH80" s="63" t="n">
+        <v>45615</v>
+      </c>
+      <c r="GJ80" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis. NPPF ref back comments from app requested 17/12</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -21679,11 +21875,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE81" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH81" s="62" t="inlineStr">
         <is>
           <t>22 and 24 St.Annes Road</t>
@@ -21738,7 +21929,10 @@
       <c r="EH81" s="63" t="n">
         <v>45674</v>
       </c>
-      <c r="EK81" s="62" t="inlineStr">
+      <c r="GH81" s="63" t="n">
+        <v>45622</v>
+      </c>
+      <c r="GJ81" s="62" t="inlineStr">
         <is>
           <t>BNG - yes - condition needed if approved. NPPF ref back not needed. 6 week challenge date 28 Feb 25</t>
         </is>
@@ -21854,11 +22048,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE82" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH82" s="62" t="inlineStr">
         <is>
           <t>87 Queenshill Road</t>
@@ -21918,13 +22107,16 @@
       <c r="EH82" s="63" t="n">
         <v>45674</v>
       </c>
-      <c r="EK82" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed.  De minimis. NPPF ref back 16 Dec 2024, comments due 6 January 2025. 6 week challenge date 28 Feb 2025</t>
-        </is>
-      </c>
       <c r="GE82" s="62" t="n">
         <v>578</v>
+      </c>
+      <c r="GH82" s="63" t="n">
+        <v>45582</v>
+      </c>
+      <c r="GJ82" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed.  De minimis. NPPF ref back 16 Dec 2024, comments due 6 January 2025. 6 week challenge date 28 Feb 2025</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -22041,11 +22233,6 @@
           <t>Nicola Robinson</t>
         </is>
       </c>
-      <c r="CE83" s="62" t="inlineStr">
-        <is>
-          <t>Nicola Robinson</t>
-        </is>
-      </c>
       <c r="CH83" s="62" t="inlineStr">
         <is>
           <t>20 Whiteladies Road</t>
@@ -22119,7 +22306,10 @@
       <c r="EH83" s="63" t="n">
         <v>45674</v>
       </c>
-      <c r="EK83" s="62" t="inlineStr">
+      <c r="GH83" s="63" t="n">
+        <v>45611</v>
+      </c>
+      <c r="GJ83" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed.  De minimis. CIL liable. NPPF ref back not needed. 6 week challenge date 28 Feb 25</t>
         </is>
@@ -22183,7 +22373,7 @@
         <v>45643</v>
       </c>
       <c r="AB84" s="63" t="n">
-        <v>45940</v>
+        <v>45959</v>
       </c>
       <c r="AC84" s="63" t="n">
         <v>45614</v>
@@ -22230,11 +22420,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE84" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CG84" s="62" t="inlineStr">
         <is>
           <t>Rebecca due to CIL issue</t>
@@ -22307,13 +22492,16 @@
       <c r="EH84" s="63" t="n">
         <v>45688</v>
       </c>
-      <c r="EK84" s="62" t="inlineStr">
-        <is>
-          <t>BNG condition applies if approved. CIL liable. NPPF ref back not needed 6 week challenge date 14 March 2025</t>
-        </is>
-      </c>
       <c r="GE84" s="62" t="n">
         <v>2826.03</v>
+      </c>
+      <c r="GH84" s="63" t="n">
+        <v>45614</v>
+      </c>
+      <c r="GJ84" s="62" t="inlineStr">
+        <is>
+          <t>BNG condition applies if approved. CIL liable. NPPF ref back not needed 6 week challenge date 14 March 2025</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -22424,12 +22612,12 @@
       </c>
       <c r="BX85" s="62" t="inlineStr">
         <is>
-          <t>Gareth Fort (Nichola Robinson validated)</t>
-        </is>
-      </c>
-      <c r="CE85" s="62" t="inlineStr">
-        <is>
-          <t>Gareth Fort (Nichola Robinson validated)</t>
+          <t>Nichola Robinson (v)</t>
+        </is>
+      </c>
+      <c r="BZ85" s="62" t="inlineStr">
+        <is>
+          <t>Gareth Fort</t>
         </is>
       </c>
       <c r="CH85" s="62" t="inlineStr">
@@ -22509,13 +22697,16 @@
       <c r="EH85" s="63" t="n">
         <v>45688</v>
       </c>
-      <c r="EK85" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis. NPPF ref back not needed. 6 week challenge date 14 March 2025</t>
-        </is>
-      </c>
       <c r="GE85" s="62" t="n">
         <v>1535</v>
+      </c>
+      <c r="GH85" s="63" t="n">
+        <v>45643</v>
+      </c>
+      <c r="GJ85" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis. NPPF ref back not needed. 6 week challenge date 14 March 2025</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -22593,11 +22784,6 @@
           <t>Graham Wraight</t>
         </is>
       </c>
-      <c r="CE86" s="62" t="inlineStr">
-        <is>
-          <t>Graham Wraight</t>
-        </is>
-      </c>
       <c r="CH86" s="62" t="inlineStr">
         <is>
           <t>10 Rylestone Grove</t>
@@ -22642,7 +22828,7 @@
       <c r="EA86" s="63" t="n">
         <v>45587</v>
       </c>
-      <c r="EK86" s="62" t="inlineStr">
+      <c r="GJ86" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">App says BNG exempt (self build). CIL Liable. Application closed down 26 Feb 2025 due to no response to invalid letter and chaser emails. </t>
         </is>
@@ -22723,11 +22909,6 @@
           <t>Jonathan Edwards</t>
         </is>
       </c>
-      <c r="CE87" s="62" t="inlineStr">
-        <is>
-          <t>Jonathan Edwards</t>
-        </is>
-      </c>
       <c r="CH87" s="62" t="inlineStr">
         <is>
           <t>65 Lodge Causeway</t>
@@ -22779,7 +22960,7 @@
       <c r="EA87" s="63" t="n">
         <v>45694</v>
       </c>
-      <c r="EK87" s="62" t="inlineStr">
+      <c r="GJ87" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. Applicant has decided not to proceed</t>
         </is>
@@ -22893,11 +23074,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE88" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH88" s="62" t="inlineStr">
         <is>
           <t>Colne Spring Villa</t>
@@ -22957,13 +23133,16 @@
       <c r="EH88" s="63" t="n">
         <v>45728</v>
       </c>
-      <c r="EK88" s="62" t="inlineStr">
-        <is>
-          <t>BNG condition applies if approved. 6 week date 23 April 2025</t>
-        </is>
-      </c>
       <c r="GE88" s="62" t="n">
         <v>5202</v>
+      </c>
+      <c r="GH88" s="63" t="n">
+        <v>45678</v>
+      </c>
+      <c r="GJ88" s="62" t="inlineStr">
+        <is>
+          <t>BNG condition applies if approved. 6 week date 23 April 2025</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -23074,11 +23253,6 @@
           <t>Graham Wraight</t>
         </is>
       </c>
-      <c r="CE89" s="62" t="inlineStr">
-        <is>
-          <t>Graham Wraight</t>
-        </is>
-      </c>
       <c r="CG89" s="62" t="inlineStr">
         <is>
           <t>Rebecca</t>
@@ -23141,7 +23315,10 @@
       <c r="EH89" s="63" t="n">
         <v>45729</v>
       </c>
-      <c r="EK89" s="62" t="inlineStr">
+      <c r="GH89" s="63" t="n">
+        <v>45677</v>
+      </c>
+      <c r="GJ89" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. Self build. CIL liable. NPPF comments requested before starting. 6 week date 24 April 2025</t>
         </is>
@@ -23255,11 +23432,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE90" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH90" s="62" t="inlineStr">
         <is>
           <t>14 Marlborough Street</t>
@@ -23319,7 +23491,10 @@
       <c r="EH90" s="63" t="n">
         <v>45749</v>
       </c>
-      <c r="EK90" s="62" t="inlineStr">
+      <c r="GH90" s="63" t="n">
+        <v>45714</v>
+      </c>
+      <c r="GJ90" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -23431,11 +23606,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE91" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH91" s="62" t="inlineStr">
         <is>
           <t>515-517</t>
@@ -23508,7 +23678,10 @@
       <c r="EH91" s="63" t="n">
         <v>45761</v>
       </c>
-      <c r="EK91" s="62" t="inlineStr">
+      <c r="GH91" s="63" t="n">
+        <v>45708</v>
+      </c>
+      <c r="GJ91" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -23625,11 +23798,6 @@
           <t>Claire Shearing</t>
         </is>
       </c>
-      <c r="CE92" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH92" s="62" t="inlineStr">
         <is>
           <t>Bull Inn</t>
@@ -23705,7 +23873,10 @@
       <c r="EH92" s="63" t="n">
         <v>45783</v>
       </c>
-      <c r="EK92" s="62" t="inlineStr">
+      <c r="GH92" s="63" t="n">
+        <v>45733</v>
+      </c>
+      <c r="GJ92" s="62" t="inlineStr">
         <is>
           <t>BNG condition applies if approved.</t>
         </is>
@@ -23824,11 +23995,6 @@
           <t>Zoe Raygen</t>
         </is>
       </c>
-      <c r="CE93" s="62" t="inlineStr">
-        <is>
-          <t>Rebecca Dickson / Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH93" s="62" t="inlineStr">
         <is>
           <t>Building 11</t>
@@ -23896,7 +24062,10 @@
       <c r="EH93" s="63" t="n">
         <v>45792</v>
       </c>
-      <c r="EK93" s="62" t="inlineStr">
+      <c r="GH93" s="63" t="n">
+        <v>45737</v>
+      </c>
+      <c r="GJ93" s="62" t="inlineStr">
         <is>
           <t>BNG condition applies if approved.</t>
         </is>
@@ -24010,12 +24179,12 @@
       </c>
       <c r="BX94" s="62" t="inlineStr">
         <is>
-          <t>Rebecca Dickson (Zoe Raygen)</t>
-        </is>
-      </c>
-      <c r="CE94" s="62" t="inlineStr">
-        <is>
-          <t>Rebecca Dickson (Zoe Raygen)</t>
+          <t>Rebecca Dickson</t>
+        </is>
+      </c>
+      <c r="BZ94" s="62" t="inlineStr">
+        <is>
+          <t>Zoe Raygen</t>
         </is>
       </c>
       <c r="CH94" s="62" t="inlineStr">
@@ -24088,7 +24257,10 @@
       <c r="EH94" s="63" t="n">
         <v>45796</v>
       </c>
-      <c r="EK94" s="62" t="inlineStr">
+      <c r="GH94" s="63" t="n">
+        <v>45722</v>
+      </c>
+      <c r="GJ94" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -24207,11 +24379,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE95" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH95" s="62" t="inlineStr">
         <is>
           <t>17 Clarendon Road</t>
@@ -24282,7 +24449,10 @@
       <c r="EH95" s="63" t="n">
         <v>45796</v>
       </c>
-      <c r="EK95" s="62" t="inlineStr">
+      <c r="GH95" s="63" t="n">
+        <v>45716</v>
+      </c>
+      <c r="GJ95" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -24398,11 +24568,6 @@
           <t>Bhu Thandi</t>
         </is>
       </c>
-      <c r="CE96" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH96" s="62" t="inlineStr">
         <is>
           <t>37 Sandholme Road</t>
@@ -24455,7 +24620,10 @@
       <c r="EH96" s="63" t="n">
         <v>45797</v>
       </c>
-      <c r="EK96" s="62" t="inlineStr">
+      <c r="GH96" s="63" t="n">
+        <v>45719</v>
+      </c>
+      <c r="GJ96" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -24563,17 +24731,12 @@
       </c>
       <c r="BX97" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validated</t>
+          <t>Zoe Raygen (v)</t>
         </is>
       </c>
       <c r="BZ97" s="62" t="inlineStr">
         <is>
           <t>Claire Shearing</t>
-        </is>
-      </c>
-      <c r="CE97" s="62" t="inlineStr">
-        <is>
-          <t>Zoe Raygen validated / Claire Shearing</t>
         </is>
       </c>
       <c r="CH97" s="62" t="inlineStr">
@@ -24643,7 +24806,10 @@
       <c r="EH97" s="63" t="n">
         <v>45797</v>
       </c>
-      <c r="EK97" s="62" t="inlineStr">
+      <c r="GH97" s="63" t="n">
+        <v>45744</v>
+      </c>
+      <c r="GJ97" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -24765,12 +24931,7 @@
       </c>
       <c r="BX98" s="62" t="inlineStr">
         <is>
-          <t>Jennifer Wallace (was Downs)</t>
-        </is>
-      </c>
-      <c r="CE98" s="62" t="inlineStr">
-        <is>
-          <t>Jennifer Wallace (was Downs)</t>
+          <t>Jennifer Wallace</t>
         </is>
       </c>
       <c r="CH98" s="62" t="inlineStr">
@@ -24840,7 +25001,10 @@
       <c r="EH98" s="63" t="n">
         <v>45799</v>
       </c>
-      <c r="EK98" s="62" t="inlineStr">
+      <c r="GH98" s="63" t="n">
+        <v>45747</v>
+      </c>
+      <c r="GJ98" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -24931,7 +25095,7 @@
           <t>Considerations of the size of the rear extension judged against the preservation of the special architectural or historic interest of the host building</t>
         </is>
       </c>
-      <c r="EK99" s="62" t="inlineStr">
+      <c r="GJ99" s="62" t="inlineStr">
         <is>
           <t>Householder, so returned</t>
         </is>
@@ -25049,11 +25213,6 @@
           <t>Kevin Savage</t>
         </is>
       </c>
-      <c r="CE100" s="62" t="inlineStr">
-        <is>
-          <t>Kevin Savage</t>
-        </is>
-      </c>
       <c r="CG100" s="62" t="inlineStr">
         <is>
           <t>David</t>
@@ -25116,7 +25275,10 @@
       <c r="EH100" s="63" t="n">
         <v>45813</v>
       </c>
-      <c r="EK100" s="62" t="inlineStr">
+      <c r="GH100" s="63" t="n">
+        <v>45748</v>
+      </c>
+      <c r="GJ100" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -25225,11 +25387,6 @@
           <t>Jack Hobbs</t>
         </is>
       </c>
-      <c r="CE101" s="62" t="inlineStr">
-        <is>
-          <t>Jack Hobbs</t>
-        </is>
-      </c>
       <c r="CG101" s="62" t="inlineStr">
         <is>
           <t>David</t>
@@ -25289,7 +25446,10 @@
       <c r="EH101" s="63" t="n">
         <v>45818</v>
       </c>
-      <c r="EK101" s="62" t="inlineStr">
+      <c r="GH101" s="63" t="n">
+        <v>45770</v>
+      </c>
+      <c r="GJ101" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -25421,12 +25581,7 @@
       </c>
       <c r="BX102" s="62" t="inlineStr">
         <is>
-          <t>Jennifer Wallace (was Downs)</t>
-        </is>
-      </c>
-      <c r="CE102" s="62" t="inlineStr">
-        <is>
-          <t>Jennifer Wallace (was Downs)</t>
+          <t>Jennifer Wallace</t>
         </is>
       </c>
       <c r="CG102" s="62" t="inlineStr">
@@ -25501,7 +25656,10 @@
       <c r="EH102" s="63" t="n">
         <v>45820</v>
       </c>
-      <c r="EK102" s="62" t="inlineStr">
+      <c r="GH102" s="63" t="n">
+        <v>45742</v>
+      </c>
+      <c r="GJ102" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. Self and custom build development</t>
         </is>
@@ -25612,11 +25770,6 @@
           <t>Nichola Robinson</t>
         </is>
       </c>
-      <c r="CE103" s="62" t="inlineStr">
-        <is>
-          <t>Nichola Robinson</t>
-        </is>
-      </c>
       <c r="CG103" s="62" t="inlineStr">
         <is>
           <t>checked ok to issue with David M</t>
@@ -25684,7 +25837,10 @@
       <c r="EH103" s="63" t="n">
         <v>45831</v>
       </c>
-      <c r="EK103" s="62" t="inlineStr">
+      <c r="GH103" s="63" t="n">
+        <v>45730</v>
+      </c>
+      <c r="GJ103" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -25802,11 +25958,6 @@
           <t>Jonathan Edwards</t>
         </is>
       </c>
-      <c r="CE104" s="62" t="inlineStr">
-        <is>
-          <t>Jonathan Edwards</t>
-        </is>
-      </c>
       <c r="CH104" s="62" t="inlineStr">
         <is>
           <t>No.7 Belvedere Road</t>
@@ -25874,7 +26025,10 @@
       <c r="EH104" s="63" t="n">
         <v>45832</v>
       </c>
-      <c r="EK104" s="62" t="inlineStr">
+      <c r="GH104" s="63" t="n">
+        <v>45783</v>
+      </c>
+      <c r="GJ104" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -25974,11 +26128,8 @@
       </c>
       <c r="BX105" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY105" s="63" t="n">
-        <v>45784</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ105" s="62" t="inlineStr">
         <is>
@@ -25988,11 +26139,6 @@
       <c r="CA105" s="63" t="n">
         <v>45784</v>
       </c>
-      <c r="CE105" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH105" s="62" t="inlineStr">
         <is>
           <t>Flat 4</t>
@@ -26060,7 +26206,10 @@
       <c r="EH105" s="63" t="n">
         <v>45835</v>
       </c>
-      <c r="EK105" s="62" t="inlineStr">
+      <c r="GH105" s="63" t="n">
+        <v>45792</v>
+      </c>
+      <c r="GJ105" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -26179,17 +26328,12 @@
       </c>
       <c r="BX106" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validated</t>
+          <t>Zoe Raygen (v)</t>
         </is>
       </c>
       <c r="BZ106" s="62" t="inlineStr">
         <is>
           <t>Claire Shearing</t>
-        </is>
-      </c>
-      <c r="CE106" s="62" t="inlineStr">
-        <is>
-          <t>Zoe Raygen validated / Claire Shearing</t>
         </is>
       </c>
       <c r="CH106" s="62" t="inlineStr">
@@ -26264,7 +26408,10 @@
       <c r="EH106" s="63" t="n">
         <v>45835</v>
       </c>
-      <c r="EK106" s="62" t="inlineStr">
+      <c r="GH106" s="63" t="n">
+        <v>45789</v>
+      </c>
+      <c r="GJ106" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -26376,7 +26523,7 @@
       </c>
       <c r="BX107" s="62" t="inlineStr">
         <is>
-          <t>Gareth Fort Rebecca Dickson</t>
+          <t>Rebecca Dickson</t>
         </is>
       </c>
       <c r="BY107" s="63" t="n">
@@ -26390,11 +26537,6 @@
       <c r="CA107" s="63" t="n">
         <v>45776</v>
       </c>
-      <c r="CE107" s="62" t="inlineStr">
-        <is>
-          <t>Gareth Fort Rebecca Dickson / Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH107" s="62" t="inlineStr">
         <is>
           <t>6 Gordon Road</t>
@@ -26467,7 +26609,10 @@
       <c r="EH107" s="63" t="n">
         <v>45835</v>
       </c>
-      <c r="EK107" s="62" t="inlineStr">
+      <c r="GH107" s="63" t="n">
+        <v>45786</v>
+      </c>
+      <c r="GJ107" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -26584,11 +26729,6 @@
       <c r="BY108" s="63" t="n">
         <v>45778</v>
       </c>
-      <c r="CE108" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH108" s="62" t="inlineStr">
         <is>
           <t>87A Redland Road</t>
@@ -26661,7 +26801,10 @@
       <c r="EH108" s="63" t="n">
         <v>45839</v>
       </c>
-      <c r="EK108" s="62" t="inlineStr">
+      <c r="GH108" s="63" t="n">
+        <v>45791</v>
+      </c>
+      <c r="GJ108" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -26778,11 +26921,6 @@
       <c r="BY109" s="63" t="n">
         <v>45784</v>
       </c>
-      <c r="CE109" s="62" t="inlineStr">
-        <is>
-          <t>Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH109" s="62" t="inlineStr">
         <is>
           <t>No. 6 Tyndalls Park Road</t>
@@ -26848,7 +26986,10 @@
       <c r="EH109" s="63" t="n">
         <v>45840</v>
       </c>
-      <c r="EK109" s="62" t="inlineStr">
+      <c r="GH109" s="63" t="n">
+        <v>45797</v>
+      </c>
+      <c r="GJ109" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -26955,11 +27096,6 @@
       <c r="BY110" s="63" t="n">
         <v>45800</v>
       </c>
-      <c r="CE110" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH110" s="62" t="inlineStr">
         <is>
           <t>11-13 High Street</t>
@@ -27030,7 +27166,10 @@
       <c r="EH110" s="63" t="n">
         <v>45855</v>
       </c>
-      <c r="EK110" s="62" t="inlineStr">
+      <c r="GH110" s="63" t="n">
+        <v>45814</v>
+      </c>
+      <c r="GJ110" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -27125,11 +27264,8 @@
       </c>
       <c r="BX111" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY111" s="63" t="n">
-        <v>45833</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ111" s="62" t="inlineStr">
         <is>
@@ -27139,11 +27275,6 @@
       <c r="CA111" s="63" t="n">
         <v>45833</v>
       </c>
-      <c r="CE111" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH111" s="62" t="inlineStr">
         <is>
           <t>237/237A Gloucester Road</t>
@@ -27200,7 +27331,10 @@
       <c r="EH111" s="63" t="n">
         <v>45861</v>
       </c>
-      <c r="EK111" s="62" t="inlineStr">
+      <c r="GH111" s="63" t="n">
+        <v>45824</v>
+      </c>
+      <c r="GJ111" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -27312,11 +27446,8 @@
       </c>
       <c r="BX112" s="62" t="inlineStr">
         <is>
-          <t>Andrew Robinson validating</t>
-        </is>
-      </c>
-      <c r="BY112" s="63" t="n">
-        <v>45860</v>
+          <t>Andrew Robinson (v)</t>
+        </is>
       </c>
       <c r="BZ112" s="62" t="inlineStr">
         <is>
@@ -27326,11 +27457,6 @@
       <c r="CA112" s="63" t="n">
         <v>45860</v>
       </c>
-      <c r="CE112" s="62" t="inlineStr">
-        <is>
-          <t>Andrew Robinson validating / Cullum Parker</t>
-        </is>
-      </c>
       <c r="CH112" s="62" t="inlineStr">
         <is>
           <t>7 Redcatch Road</t>
@@ -27398,7 +27524,10 @@
       <c r="EH112" s="63" t="n">
         <v>45870</v>
       </c>
-      <c r="EK112" s="62" t="inlineStr">
+      <c r="GH112" s="63" t="n">
+        <v>45839</v>
+      </c>
+      <c r="GJ112" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -27504,16 +27633,11 @@
       </c>
       <c r="BX113" s="62" t="inlineStr">
         <is>
-          <t>Jennifer Wallace Claire Shearing</t>
+          <t>Claire Shearing</t>
         </is>
       </c>
       <c r="BY113" s="63" t="n">
         <v>45833</v>
-      </c>
-      <c r="CE113" s="62" t="inlineStr">
-        <is>
-          <t>Jennifer Wallace Claire Shearing</t>
-        </is>
       </c>
       <c r="CH113" s="62" t="inlineStr">
         <is>
@@ -27579,13 +27703,16 @@
       <c r="EH113" s="63" t="n">
         <v>45876</v>
       </c>
-      <c r="EK113" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis</t>
-        </is>
-      </c>
       <c r="GE113" s="62" t="n">
         <v>3468</v>
+      </c>
+      <c r="GH113" s="63" t="n">
+        <v>45826</v>
+      </c>
+      <c r="GJ113" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -27688,11 +27815,8 @@
       </c>
       <c r="BX114" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY114" s="63" t="n">
-        <v>45860</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ114" s="62" t="inlineStr">
         <is>
@@ -27702,11 +27826,6 @@
       <c r="CA114" s="63" t="n">
         <v>45860</v>
       </c>
-      <c r="CE114" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Cullum Parker</t>
-        </is>
-      </c>
       <c r="CH114" s="62" t="inlineStr">
         <is>
           <t>The Annexe at 11-13 Whiteladies Road</t>
@@ -27772,13 +27891,16 @@
       <c r="EH114" s="63" t="n">
         <v>45877</v>
       </c>
-      <c r="EK114" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis</t>
-        </is>
-      </c>
       <c r="GE114" s="62" t="n">
         <v>3025</v>
+      </c>
+      <c r="GH114" s="63" t="n">
+        <v>45842</v>
+      </c>
+      <c r="GJ114" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -27900,11 +28022,8 @@
       </c>
       <c r="BX115" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY115" s="63" t="n">
-        <v>45784</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ115" s="62" t="inlineStr">
         <is>
@@ -27914,11 +28033,6 @@
       <c r="CA115" s="63" t="n">
         <v>45784</v>
       </c>
-      <c r="CE115" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Bhu Thandi</t>
-        </is>
-      </c>
       <c r="CH115" s="62" t="inlineStr">
         <is>
           <t>No. 9 Priory Road</t>
@@ -27989,7 +28103,10 @@
       <c r="EH115" s="63" t="n">
         <v>45889</v>
       </c>
-      <c r="EK115" s="62" t="inlineStr">
+      <c r="GH115" s="63" t="n">
+        <v>45797</v>
+      </c>
+      <c r="GJ115" s="62" t="inlineStr">
         <is>
           <t>BNG condition applies if approved</t>
         </is>
@@ -28063,11 +28180,6 @@
       <c r="BY116" s="63" t="n">
         <v>45911</v>
       </c>
-      <c r="CE116" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH116" s="62" t="inlineStr">
         <is>
           <t>Unit 7 Newbridge Trading Estate</t>
@@ -28121,7 +28233,7 @@
       <c r="DZ116" s="62" t="n">
         <v>588</v>
       </c>
-      <c r="EK116" s="62" t="inlineStr">
+      <c r="GJ116" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -28233,11 +28345,6 @@
       <c r="BY117" s="63" t="n">
         <v>45853</v>
       </c>
-      <c r="CE117" s="62" t="inlineStr">
-        <is>
-          <t>Jack Hobbs</t>
-        </is>
-      </c>
       <c r="CG117" s="62" t="inlineStr">
         <is>
           <t>David?</t>
@@ -28305,7 +28412,10 @@
       <c r="EH117" s="63" t="n">
         <v>45926</v>
       </c>
-      <c r="EK117" s="62" t="inlineStr">
+      <c r="GH117" s="63" t="n">
+        <v>45874</v>
+      </c>
+      <c r="GJ117" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -28370,11 +28480,6 @@
       <c r="BY118" s="63" t="n">
         <v>45917</v>
       </c>
-      <c r="CE118" s="62" t="inlineStr">
-        <is>
-          <t>Hayley Butcher</t>
-        </is>
-      </c>
       <c r="CH118" s="62" t="inlineStr">
         <is>
           <t>1-3 High Street</t>
@@ -28414,7 +28519,7 @@
       <c r="DZ118" s="62" t="n">
         <v>1176</v>
       </c>
-      <c r="EK118" s="62" t="inlineStr">
+      <c r="GJ118" s="62" t="inlineStr">
         <is>
           <t>Withdrawn 01/10/2025</t>
         </is>
@@ -28528,11 +28633,8 @@
       </c>
       <c r="BX119" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY119" s="63" t="n">
-        <v>45903</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ119" s="62" t="inlineStr">
         <is>
@@ -28541,11 +28643,6 @@
       </c>
       <c r="CA119" s="63" t="n">
         <v>45903</v>
-      </c>
-      <c r="CE119" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Zoe Raygen</t>
-        </is>
       </c>
       <c r="CH119" s="62" t="inlineStr">
         <is>
@@ -28611,13 +28708,16 @@
       <c r="EH119" s="63" t="n">
         <v>45937</v>
       </c>
-      <c r="EK119" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis</t>
-        </is>
-      </c>
       <c r="GE119" s="62" t="n">
         <v>528</v>
+      </c>
+      <c r="GH119" s="63" t="n">
+        <v>45880</v>
+      </c>
+      <c r="GJ119" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -28729,11 +28829,8 @@
       </c>
       <c r="BX120" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY120" s="63" t="n">
-        <v>45903</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ120" s="62" t="inlineStr">
         <is>
@@ -28743,11 +28840,6 @@
       <c r="CA120" s="63" t="n">
         <v>45903</v>
       </c>
-      <c r="CE120" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH120" s="62" t="inlineStr">
         <is>
           <t>Chasefield House</t>
@@ -28824,7 +28916,10 @@
       <c r="EH120" s="63" t="n">
         <v>45938</v>
       </c>
-      <c r="EK120" s="62" t="inlineStr">
+      <c r="GH120" s="63" t="n">
+        <v>45874</v>
+      </c>
+      <c r="GJ120" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -28935,11 +29030,6 @@
       <c r="BY121" s="63" t="n">
         <v>45876</v>
       </c>
-      <c r="CE121" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH121" s="62" t="inlineStr">
         <is>
           <t>144 Whitehall Road</t>
@@ -28994,7 +29084,10 @@
       <c r="EH121" s="63" t="n">
         <v>45937</v>
       </c>
-      <c r="EK121" s="62" t="inlineStr">
+      <c r="GH121" s="63" t="n">
+        <v>45884</v>
+      </c>
+      <c r="GJ121" s="62" t="inlineStr">
         <is>
           <t>fee rec late PM so valid date from next day</t>
         </is>
@@ -29105,11 +29198,6 @@
       <c r="BY122" s="63" t="n">
         <v>45876</v>
       </c>
-      <c r="CE122" s="62" t="inlineStr">
-        <is>
-          <t>Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH122" s="62" t="inlineStr">
         <is>
           <t>144 Whitehall Road</t>
@@ -29167,7 +29255,10 @@
       <c r="EH122" s="63" t="n">
         <v>45937</v>
       </c>
-      <c r="EK122" s="62" t="inlineStr">
+      <c r="GH122" s="63" t="n">
+        <v>45884</v>
+      </c>
+      <c r="GJ122" s="62" t="inlineStr">
         <is>
           <t>fee rec late PM so valid date from next day</t>
         </is>
@@ -29274,11 +29365,8 @@
       </c>
       <c r="BX123" s="62" t="inlineStr">
         <is>
-          <t>Darren Hendley validating</t>
-        </is>
-      </c>
-      <c r="BY123" s="63" t="n">
-        <v>45884</v>
+          <t>Darren Hendley (v)</t>
+        </is>
       </c>
       <c r="BZ123" s="62" t="inlineStr">
         <is>
@@ -29288,11 +29376,6 @@
       <c r="CA123" s="63" t="n">
         <v>45884</v>
       </c>
-      <c r="CE123" s="62" t="inlineStr">
-        <is>
-          <t>Darren Hendley validating / Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH123" s="62" t="inlineStr">
         <is>
           <t>110-112 The Assembly</t>
@@ -29365,13 +29448,16 @@
       <c r="EH123" s="63" t="n">
         <v>45947</v>
       </c>
-      <c r="EK123" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis. EoT needed due to certs update</t>
-        </is>
-      </c>
       <c r="GE123" s="62" t="n">
         <v>588</v>
+      </c>
+      <c r="GH123" s="63" t="n">
+        <v>45883</v>
+      </c>
+      <c r="GJ123" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis. EoT needed due to certs update</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -29486,11 +29572,6 @@
       <c r="BY124" s="63" t="n">
         <v>45887</v>
       </c>
-      <c r="CE124" s="62" t="inlineStr">
-        <is>
-          <t>Zoe Raygen</t>
-        </is>
-      </c>
       <c r="CH124" s="62" t="inlineStr">
         <is>
           <t>11-13 Whiteladies Road</t>
@@ -29553,7 +29634,10 @@
       <c r="EH124" s="63" t="n">
         <v>45960</v>
       </c>
-      <c r="EK124" s="62" t="inlineStr">
+      <c r="GH124" s="63" t="n">
+        <v>45895</v>
+      </c>
+      <c r="GJ124" s="62" t="inlineStr">
         <is>
           <t>10 days notice not given. BNG exemption claimed. De minimis</t>
         </is>
@@ -29659,11 +29743,6 @@
       <c r="BY125" s="63" t="n">
         <v>45911</v>
       </c>
-      <c r="CE125" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH125" s="62" t="inlineStr">
         <is>
           <t>13 Risdale Road</t>
@@ -29721,7 +29800,10 @@
       <c r="EH125" s="63" t="n">
         <v>45967</v>
       </c>
-      <c r="EK125" s="62" t="inlineStr">
+      <c r="GH125" s="63" t="n">
+        <v>45929</v>
+      </c>
+      <c r="GJ125" s="62" t="inlineStr">
         <is>
           <t>BNG condition if approved</t>
         </is>
@@ -29838,11 +29920,6 @@
       <c r="BY126" s="63" t="n">
         <v>45916</v>
       </c>
-      <c r="CE126" s="62" t="inlineStr">
-        <is>
-          <t>Tom Gilbert-Wooldridge</t>
-        </is>
-      </c>
       <c r="CH126" s="62" t="inlineStr">
         <is>
           <t>2–5 Highland Square</t>
@@ -29910,7 +29987,10 @@
       <c r="EH126" s="63" t="n">
         <v>45979</v>
       </c>
-      <c r="EK126" s="62" t="inlineStr">
+      <c r="GH126" s="63" t="n">
+        <v>45931</v>
+      </c>
+      <c r="GJ126" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -30030,11 +30110,6 @@
       <c r="CA127" s="63" t="n">
         <v>45888</v>
       </c>
-      <c r="CE127" s="62" t="inlineStr">
-        <is>
-          <t>Gareth Fort / Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH127" s="62" t="inlineStr">
         <is>
           <t>23 Hillsborough Rd</t>
@@ -30089,7 +30164,10 @@
       <c r="EH127" s="63" t="n">
         <v>45982</v>
       </c>
-      <c r="EK127" s="62" t="inlineStr">
+      <c r="GH127" s="63" t="n">
+        <v>45938</v>
+      </c>
+      <c r="GJ127" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">BNG exemption claimed. De minimis. </t>
         </is>
@@ -30203,11 +30281,6 @@
       <c r="CA128" s="63" t="n">
         <v>45923</v>
       </c>
-      <c r="CE128" s="62" t="inlineStr">
-        <is>
-          <t>George Baird / Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH128" s="62" t="inlineStr">
         <is>
           <t>6-8 Emery Road</t>
@@ -30267,7 +30340,10 @@
       <c r="EH128" s="63" t="n">
         <v>45987</v>
       </c>
-      <c r="EK128" s="62" t="inlineStr">
+      <c r="GH128" s="63" t="n">
+        <v>45938</v>
+      </c>
+      <c r="GJ128" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -30335,7 +30411,7 @@
         <v>45944</v>
       </c>
       <c r="AE129" s="63" t="n">
-        <v>45974</v>
+        <v>45961</v>
       </c>
       <c r="AF129" s="63" t="n">
         <v>45974</v>
@@ -30376,11 +30452,8 @@
       </c>
       <c r="BX129" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validating</t>
-        </is>
-      </c>
-      <c r="BY129" s="63" t="n">
-        <v>45922</v>
+          <t>Zoe Raygen (v)</t>
+        </is>
       </c>
       <c r="BZ129" s="62" t="inlineStr">
         <is>
@@ -30390,11 +30463,6 @@
       <c r="CA129" s="63" t="n">
         <v>45922</v>
       </c>
-      <c r="CE129" s="62" t="inlineStr">
-        <is>
-          <t>Zoe Raygen validating/ Gareth Fort</t>
-        </is>
-      </c>
       <c r="CH129" s="62" t="inlineStr">
         <is>
           <t>286 - 292 Wells Road</t>
@@ -30462,7 +30530,10 @@
       <c r="EH129" s="63" t="n">
         <v>45993</v>
       </c>
-      <c r="EK129" s="62" t="inlineStr">
+      <c r="GH129" s="63" t="n">
+        <v>45912</v>
+      </c>
+      <c r="GJ129" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -30568,11 +30639,8 @@
       </c>
       <c r="BX130" s="62" t="inlineStr">
         <is>
-          <t>Zoe Raygen validating</t>
-        </is>
-      </c>
-      <c r="BY130" s="63" t="n">
-        <v>45950</v>
+          <t>Zoe Raygen (v)</t>
+        </is>
       </c>
       <c r="BZ130" s="62" t="inlineStr">
         <is>
@@ -30582,11 +30650,6 @@
       <c r="CA130" s="63" t="n">
         <v>45950</v>
       </c>
-      <c r="CE130" s="62" t="inlineStr">
-        <is>
-          <t>Zoe Raygen validating / Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH130" s="62" t="inlineStr">
         <is>
           <t>61 Cotman Walk</t>
@@ -30644,7 +30707,10 @@
       <c r="EH130" s="63" t="n">
         <v>45993</v>
       </c>
-      <c r="EK130" s="62" t="inlineStr">
+      <c r="GH130" s="63" t="n">
+        <v>45946</v>
+      </c>
+      <c r="GJ130" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -30756,11 +30822,6 @@
       <c r="BY131" s="63" t="n">
         <v>45917</v>
       </c>
-      <c r="CE131" s="62" t="inlineStr">
-        <is>
-          <t>Hayley Butcher</t>
-        </is>
-      </c>
       <c r="CH131" s="62" t="inlineStr">
         <is>
           <t>16 Elmgrove Road</t>
@@ -30815,7 +30876,10 @@
       <c r="EH131" s="63" t="n">
         <v>46003</v>
       </c>
-      <c r="EK131" s="62" t="inlineStr">
+      <c r="GH131" s="63" t="n">
+        <v>45960</v>
+      </c>
+      <c r="GJ131" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -30921,11 +30985,8 @@
       </c>
       <c r="BX132" s="62" t="inlineStr">
         <is>
-          <t>Dominic Young validating</t>
-        </is>
-      </c>
-      <c r="BY132" s="63" t="n">
-        <v>45972</v>
+          <t>Dominic Young (v)</t>
+        </is>
       </c>
       <c r="BZ132" s="62" t="inlineStr">
         <is>
@@ -30935,11 +30996,6 @@
       <c r="CA132" s="63" t="n">
         <v>45972</v>
       </c>
-      <c r="CE132" s="62" t="inlineStr">
-        <is>
-          <t>Dominic Young validating / Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH132" s="62" t="inlineStr">
         <is>
           <t>Cotham School</t>
@@ -31012,7 +31068,10 @@
       <c r="EH132" s="63" t="n">
         <v>46006</v>
       </c>
-      <c r="EK132" s="62" t="inlineStr">
+      <c r="GH132" s="63" t="n">
+        <v>45967</v>
+      </c>
+      <c r="GJ132" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -31109,11 +31168,8 @@
       </c>
       <c r="BX133" s="62" t="inlineStr">
         <is>
-          <t>Dominic Young validating</t>
-        </is>
-      </c>
-      <c r="BY133" s="63" t="n">
-        <v>45972</v>
+          <t>Dominic Young (v)</t>
+        </is>
       </c>
       <c r="BZ133" s="62" t="inlineStr">
         <is>
@@ -31123,11 +31179,6 @@
       <c r="CA133" s="63" t="n">
         <v>45972</v>
       </c>
-      <c r="CE133" s="62" t="inlineStr">
-        <is>
-          <t>Dominic Young validating / Jack Hobbs</t>
-        </is>
-      </c>
       <c r="CH133" s="62" t="inlineStr">
         <is>
           <t>2 Merton Road</t>
@@ -31185,7 +31236,10 @@
       <c r="EH133" s="63" t="n">
         <v>46014</v>
       </c>
-      <c r="EK133" s="62" t="inlineStr">
+      <c r="GH133" s="63" t="n">
+        <v>45965</v>
+      </c>
+      <c r="GJ133" s="62" t="inlineStr">
         <is>
           <t>resubmission of 0090</t>
         </is>
@@ -31296,11 +31350,8 @@
       </c>
       <c r="BX134" s="62" t="inlineStr">
         <is>
-          <t>Dominic Young validating</t>
-        </is>
-      </c>
-      <c r="BY134" s="63" t="n">
-        <v>45972</v>
+          <t>Dominic Young (v)</t>
+        </is>
       </c>
       <c r="BZ134" s="62" t="inlineStr">
         <is>
@@ -31310,11 +31361,6 @@
       <c r="CA134" s="63" t="n">
         <v>45972</v>
       </c>
-      <c r="CE134" s="62" t="inlineStr">
-        <is>
-          <t>Dominic Young validating / Jack Hobbs</t>
-        </is>
-      </c>
       <c r="CH134" s="62" t="inlineStr">
         <is>
           <t>Land on South West side of Strathmore Road</t>
@@ -31374,7 +31420,10 @@
       <c r="EH134" s="63" t="n">
         <v>46020</v>
       </c>
-      <c r="EK134" s="62" t="inlineStr">
+      <c r="GH134" s="63" t="n">
+        <v>45974</v>
+      </c>
+      <c r="GJ134" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -31471,11 +31520,8 @@
       </c>
       <c r="BX135" s="62" t="inlineStr">
         <is>
-          <t>Dominic Young validating</t>
-        </is>
-      </c>
-      <c r="BY135" s="63" t="n">
-        <v>45972</v>
+          <t>Dominic Young (v)</t>
+        </is>
       </c>
       <c r="BZ135" s="62" t="inlineStr">
         <is>
@@ -31490,16 +31536,6 @@
           <t>Sarah</t>
         </is>
       </c>
-      <c r="CE135" s="62" t="inlineStr">
-        <is>
-          <t>Dominic Young validating / Claire Shearing</t>
-        </is>
-      </c>
-      <c r="CF135" s="62" t="inlineStr">
-        <is>
-          <t>Sarah</t>
-        </is>
-      </c>
       <c r="CH135" s="62" t="inlineStr">
         <is>
           <t>11-13 Whiteladies Road</t>
@@ -31536,7 +31572,7 @@
         </is>
       </c>
       <c r="DC135" s="62" t="n">
-        <v>2025</v>
+        <v>100</v>
       </c>
       <c r="DQ135" s="62" t="n">
         <v>507.47</v>
@@ -31565,13 +31601,16 @@
       <c r="EH135" s="63" t="n">
         <v>46024</v>
       </c>
-      <c r="EK135" s="62" t="inlineStr">
-        <is>
-          <t>BNG exemption claimed. De minimis. No NPPF</t>
-        </is>
-      </c>
       <c r="GE135" s="62" t="n">
         <v>5292</v>
+      </c>
+      <c r="GH135" s="63" t="n">
+        <v>45972</v>
+      </c>
+      <c r="GJ135" s="62" t="inlineStr">
+        <is>
+          <t>BNG exemption claimed. De minimis. No NPPF</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -31685,11 +31724,6 @@
       <c r="BY136" s="63" t="n">
         <v>45974</v>
       </c>
-      <c r="CE136" s="62" t="inlineStr">
-        <is>
-          <t>Nichola Robinson</t>
-        </is>
-      </c>
       <c r="CH136" s="62" t="inlineStr">
         <is>
           <t>66-70 Church Road</t>
@@ -31747,7 +31781,10 @@
       <c r="EH136" s="63" t="n">
         <v>46028</v>
       </c>
-      <c r="EK136" s="62" t="inlineStr">
+      <c r="GH136" s="63" t="n">
+        <v>45981</v>
+      </c>
+      <c r="GJ136" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. No NPPF</t>
         </is>
@@ -31863,11 +31900,6 @@
       </c>
       <c r="BY137" s="63" t="n">
         <v>45974</v>
-      </c>
-      <c r="CE137" s="62" t="inlineStr">
-        <is>
-          <t>Nichola Robinson</t>
-        </is>
       </c>
       <c r="CH137" s="62" t="inlineStr">
         <is>
@@ -31933,7 +31965,10 @@
       <c r="EH137" s="63" t="n">
         <v>46030</v>
       </c>
-      <c r="EK137" s="62" t="inlineStr">
+      <c r="GH137" s="63" t="n">
+        <v>45987</v>
+      </c>
+      <c r="GJ137" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. No NPPF</t>
         </is>
@@ -32039,11 +32074,8 @@
       </c>
       <c r="BX138" s="62" t="inlineStr">
         <is>
-          <t>Dominic Young validating</t>
-        </is>
-      </c>
-      <c r="BY138" s="63" t="n">
-        <v>45972</v>
+          <t>Dominic Young (v)</t>
+        </is>
       </c>
       <c r="BZ138" s="62" t="inlineStr">
         <is>
@@ -32053,11 +32085,6 @@
       <c r="CA138" s="63" t="n">
         <v>45972</v>
       </c>
-      <c r="CE138" s="62" t="inlineStr">
-        <is>
-          <t>Dominic Young validating / Claire Shearing</t>
-        </is>
-      </c>
       <c r="CH138" s="62" t="inlineStr">
         <is>
           <t>Stoke Lodge Playing Fields</t>
@@ -32130,7 +32157,10 @@
       <c r="EH138" s="63" t="n">
         <v>46031</v>
       </c>
-      <c r="EK138" s="62" t="inlineStr">
+      <c r="GH138" s="63" t="n">
+        <v>45968</v>
+      </c>
+      <c r="GJ138" s="62" t="inlineStr">
         <is>
           <t>BNG condition if approved. No NPPF</t>
         </is>
@@ -32230,11 +32260,8 @@
       </c>
       <c r="BX139" s="62" t="inlineStr">
         <is>
-          <t>Cullum Parker validated</t>
-        </is>
-      </c>
-      <c r="BY139" s="63" t="n">
-        <v>45985</v>
+          <t>Cullum Parker (v)</t>
+        </is>
       </c>
       <c r="BZ139" s="62" t="inlineStr">
         <is>
@@ -32244,11 +32271,6 @@
       <c r="CA139" s="63" t="n">
         <v>45985</v>
       </c>
-      <c r="CE139" s="62" t="inlineStr">
-        <is>
-          <t>Cullum Parker validated / Owen Woodwards</t>
-        </is>
-      </c>
       <c r="CH139" s="62" t="inlineStr">
         <is>
           <t>26 Sturdon Road</t>
@@ -32303,7 +32325,10 @@
       <c r="EH139" s="63" t="n">
         <v>46036</v>
       </c>
-      <c r="EK139" s="62" t="inlineStr">
+      <c r="GH139" s="63" t="n">
+        <v>45988</v>
+      </c>
+      <c r="GJ139" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. No NPPF</t>
         </is>
@@ -32431,11 +32456,6 @@
       <c r="BY140" s="63" t="n">
         <v>45999</v>
       </c>
-      <c r="CE140" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Katie McDonald </t>
-        </is>
-      </c>
       <c r="CH140" s="62" t="inlineStr">
         <is>
           <t>36 Hampton Park</t>
@@ -32501,7 +32521,10 @@
       <c r="EH140" s="63" t="n">
         <v>46037</v>
       </c>
-      <c r="EK140" s="62" t="inlineStr">
+      <c r="GH140" s="63" t="n">
+        <v>46000</v>
+      </c>
+      <c r="GJ140" s="62" t="inlineStr">
         <is>
           <t>BNG condition if approved. No NPPF</t>
         </is>
@@ -32626,11 +32649,6 @@
       <c r="CA141" s="63" t="n">
         <v>45929</v>
       </c>
-      <c r="CE141" s="62" t="inlineStr">
-        <is>
-          <t>Scott Wilson (APO) / Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH141" s="62" t="inlineStr">
         <is>
           <t>Second Floor Flat 224 Bath Road</t>
@@ -32690,7 +32708,10 @@
       <c r="EH141" s="63" t="n">
         <v>46038</v>
       </c>
-      <c r="EK141" s="62" t="inlineStr">
+      <c r="GH141" s="63" t="n">
+        <v>45992</v>
+      </c>
+      <c r="GJ141" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -32797,11 +32818,6 @@
       <c r="BY142" s="63" t="n">
         <v>45999</v>
       </c>
-      <c r="CE142" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH142" s="62" t="inlineStr">
         <is>
           <t>76a Savoy Road</t>
@@ -32856,7 +32872,10 @@
       <c r="EH142" s="63" t="n">
         <v>46042</v>
       </c>
-      <c r="EK142" s="62" t="inlineStr">
+      <c r="GH142" s="63" t="n">
+        <v>46001</v>
+      </c>
+      <c r="GJ142" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -32976,11 +32995,6 @@
       <c r="BY143" s="63" t="n">
         <v>45999</v>
       </c>
-      <c r="CE143" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH143" s="62" t="inlineStr">
         <is>
           <t>33 Brockworth Crescent</t>
@@ -33051,7 +33065,10 @@
       <c r="EH143" s="63" t="n">
         <v>46043</v>
       </c>
-      <c r="EK143" s="62" t="inlineStr">
+      <c r="GH143" s="63" t="n">
+        <v>46003</v>
+      </c>
+      <c r="GJ143" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -33152,11 +33169,8 @@
       </c>
       <c r="BX144" s="62" t="inlineStr">
         <is>
-          <t>Owen Woodwards validating</t>
-        </is>
-      </c>
-      <c r="BY144" s="63" t="n">
-        <v>45999</v>
+          <t>Owen Woodwards (v)</t>
+        </is>
       </c>
       <c r="BZ144" s="62" t="inlineStr">
         <is>
@@ -33166,11 +33180,6 @@
       <c r="CA144" s="63" t="n">
         <v>45999</v>
       </c>
-      <c r="CE144" s="62" t="inlineStr">
-        <is>
-          <t>Owen Woodwards validating / Katie McDonald</t>
-        </is>
-      </c>
       <c r="CH144" s="62" t="inlineStr">
         <is>
           <t>Castle House</t>
@@ -33233,7 +33242,10 @@
       <c r="EH144" s="63" t="n">
         <v>46050</v>
       </c>
-      <c r="EK144" s="62" t="inlineStr">
+      <c r="GH144" s="63" t="n">
+        <v>46007</v>
+      </c>
+      <c r="GJ144" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -33349,11 +33361,8 @@
       </c>
       <c r="BX145" s="62" t="inlineStr">
         <is>
-          <t>Cullum Parker validated</t>
-        </is>
-      </c>
-      <c r="BY145" s="63" t="n">
-        <v>45985</v>
+          <t>Cullum Parker (v)</t>
+        </is>
       </c>
       <c r="BZ145" s="62" t="inlineStr">
         <is>
@@ -33368,16 +33377,6 @@
           <t>Matt</t>
         </is>
       </c>
-      <c r="CE145" s="62" t="inlineStr">
-        <is>
-          <t>Cullum Parker validated / Owen Woodwards</t>
-        </is>
-      </c>
-      <c r="CF145" s="62" t="inlineStr">
-        <is>
-          <t>Matt</t>
-        </is>
-      </c>
       <c r="CH145" s="62" t="inlineStr">
         <is>
           <t>former Natwest bank at 72-74 Gloucester Road</t>
@@ -33438,7 +33437,10 @@
       <c r="EH145" s="63" t="n">
         <v>46058</v>
       </c>
-      <c r="EK145" s="62" t="inlineStr">
+      <c r="GH145" s="63" t="n">
+        <v>45987</v>
+      </c>
+      <c r="GJ145" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. DL issed late due to delays in site notice &amp; admin delays</t>
         </is>
@@ -33520,12 +33522,7 @@
       </c>
       <c r="BX146" s="62" t="inlineStr">
         <is>
-          <t>Michael Boniface validating</t>
-        </is>
-      </c>
-      <c r="CE146" s="62" t="inlineStr">
-        <is>
-          <t>Michael Boniface validating</t>
+          <t>Michael Boniface (v)</t>
         </is>
       </c>
       <c r="CH146" s="62" t="inlineStr">
@@ -33566,7 +33563,7 @@
       <c r="DZ146" s="62" t="n">
         <v>588</v>
       </c>
-      <c r="EK146" s="62" t="inlineStr">
+      <c r="GJ146" s="62" t="inlineStr">
         <is>
           <t>Due to Bristol being dedesignated on 27 January, PINS does not have jurisdiction to determine this application. Returned to applicant</t>
         </is>
@@ -33624,12 +33621,7 @@
       </c>
       <c r="BX147" s="62" t="inlineStr">
         <is>
-          <t>Michael Boniface validating</t>
-        </is>
-      </c>
-      <c r="CE147" s="62" t="inlineStr">
-        <is>
-          <t>Michael Boniface validating</t>
+          <t>Michael Boniface (v)</t>
         </is>
       </c>
       <c r="CH147" s="62" t="inlineStr">
@@ -33670,7 +33662,7 @@
       <c r="DZ147" s="62" t="n">
         <v>4704</v>
       </c>
-      <c r="EK147" s="62" t="inlineStr">
+      <c r="GJ147" s="62" t="inlineStr">
         <is>
           <t>Due to Bristol being dedesignated on 27 January, PINS does not have jurisdiction to determine this application. Returned to applicant</t>
         </is>
@@ -33782,11 +33774,8 @@
       </c>
       <c r="BX148" s="62" t="inlineStr">
         <is>
-          <t>Katie McDonald validating</t>
-        </is>
-      </c>
-      <c r="BY148" s="63" t="n">
-        <v>46030</v>
+          <t>Katie McDonald (v)</t>
+        </is>
       </c>
       <c r="BZ148" s="62" t="inlineStr">
         <is>
@@ -33796,11 +33785,6 @@
       <c r="CA148" s="63" t="n">
         <v>46030</v>
       </c>
-      <c r="CE148" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald validating / Owen Woodwards</t>
-        </is>
-      </c>
       <c r="CH148" s="62" t="inlineStr">
         <is>
           <t>16-18 Cherry Lane</t>
@@ -33868,7 +33852,10 @@
       <c r="EH148" s="63" t="n">
         <v>46062</v>
       </c>
-      <c r="EK148" s="62" t="inlineStr">
+      <c r="GH148" s="63" t="n">
+        <v>46013</v>
+      </c>
+      <c r="GJ148" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -33971,11 +33958,8 @@
       </c>
       <c r="BX149" s="62" t="inlineStr">
         <is>
-          <t>Katie McDonald validating</t>
-        </is>
-      </c>
-      <c r="BY149" s="63" t="n">
-        <v>46034</v>
+          <t>Katie McDonald (v)</t>
+        </is>
       </c>
       <c r="BZ149" s="62" t="inlineStr">
         <is>
@@ -33985,11 +33969,6 @@
       <c r="CA149" s="63" t="n">
         <v>46034</v>
       </c>
-      <c r="CE149" s="62" t="inlineStr">
-        <is>
-          <t>Katie McDonald validating / Benjamin Webb</t>
-        </is>
-      </c>
       <c r="CH149" s="62" t="inlineStr">
         <is>
           <t>No.115 Hampton Road</t>
@@ -34052,7 +34031,10 @@
       <c r="EH149" s="63" t="n">
         <v>46070</v>
       </c>
-      <c r="EK149" s="62" t="inlineStr">
+      <c r="GH149" s="63" t="n">
+        <v>46027</v>
+      </c>
+      <c r="GJ149" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -34152,11 +34134,8 @@
       </c>
       <c r="BX150" s="62" t="inlineStr">
         <is>
-          <t>Hayley Butcher validating</t>
-        </is>
-      </c>
-      <c r="BY150" s="63" t="n">
-        <v>46034</v>
+          <t>Hayley Butcher (v)</t>
+        </is>
       </c>
       <c r="BZ150" s="62" t="inlineStr">
         <is>
@@ -34166,11 +34145,6 @@
       <c r="CA150" s="63" t="n">
         <v>46034</v>
       </c>
-      <c r="CE150" s="62" t="inlineStr">
-        <is>
-          <t>Hayley Butcher validating / Benjamin Webb</t>
-        </is>
-      </c>
       <c r="CH150" s="62" t="inlineStr">
         <is>
           <t>33 Brockworth Crescent</t>
@@ -34230,7 +34204,10 @@
       <c r="EH150" s="63" t="n">
         <v>46071</v>
       </c>
-      <c r="EK150" s="62" t="inlineStr">
+      <c r="GH150" s="63" t="n">
+        <v>46031</v>
+      </c>
+      <c r="GJ150" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -34315,11 +34292,8 @@
       </c>
       <c r="BX151" s="62" t="inlineStr">
         <is>
-          <t>George Baird validating</t>
-        </is>
-      </c>
-      <c r="BY151" s="63" t="n">
-        <v>46049</v>
+          <t>George Baird (v)</t>
+        </is>
       </c>
       <c r="BZ151" s="62" t="inlineStr">
         <is>
@@ -34329,11 +34303,6 @@
       <c r="CA151" s="63" t="n">
         <v>46049</v>
       </c>
-      <c r="CE151" s="62" t="inlineStr">
-        <is>
-          <t>George Baird validating/ Nichola Robinson</t>
-        </is>
-      </c>
       <c r="CH151" s="62" t="inlineStr">
         <is>
           <t>374 Southmead Road</t>
@@ -34391,7 +34360,10 @@
       <c r="EH151" s="63" t="n">
         <v>46079</v>
       </c>
-      <c r="EK151" s="62" t="inlineStr">
+      <c r="GH151" s="63" t="n">
+        <v>46035</v>
+      </c>
+      <c r="GJ151" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -34494,11 +34466,8 @@
       </c>
       <c r="BX152" s="62" t="inlineStr">
         <is>
-          <t>George Baird validating</t>
-        </is>
-      </c>
-      <c r="BY152" s="63" t="n">
-        <v>46049</v>
+          <t>George Baird (v)</t>
+        </is>
       </c>
       <c r="BZ152" s="62" t="inlineStr">
         <is>
@@ -34508,11 +34477,6 @@
       <c r="CA152" s="63" t="n">
         <v>46049</v>
       </c>
-      <c r="CE152" s="62" t="inlineStr">
-        <is>
-          <t>George Baird validating / Benjamin Webb</t>
-        </is>
-      </c>
       <c r="CH152" s="62" t="inlineStr">
         <is>
           <t>703 Fishponds Road</t>
@@ -34575,7 +34539,10 @@
       <c r="EH152" s="63" t="n">
         <v>46090</v>
       </c>
-      <c r="EK152" s="62" t="inlineStr">
+      <c r="GH152" s="63" t="n">
+        <v>46036</v>
+      </c>
+      <c r="GJ152" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis</t>
         </is>
@@ -34676,11 +34643,8 @@
       </c>
       <c r="BX153" s="62" t="inlineStr">
         <is>
-          <t>George Baird validating</t>
-        </is>
-      </c>
-      <c r="BY153" s="63" t="n">
-        <v>46062</v>
+          <t>George Baird (v)</t>
+        </is>
       </c>
       <c r="BZ153" s="62" t="inlineStr">
         <is>
@@ -34690,11 +34654,6 @@
       <c r="CA153" s="63" t="n">
         <v>46062</v>
       </c>
-      <c r="CE153" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">George Baird validating / Heather Faulkner </t>
-        </is>
-      </c>
       <c r="CG153" s="62" t="inlineStr">
         <is>
           <t>Owen</t>
@@ -34772,7 +34731,10 @@
       <c r="EH153" s="63" t="n">
         <v>46097</v>
       </c>
-      <c r="EK153" s="62" t="inlineStr">
+      <c r="GH153" s="63" t="n">
+        <v>46041</v>
+      </c>
+      <c r="GJ153" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. Missed DL target due to using last cases for new Insps in training</t>
         </is>
@@ -34876,11 +34838,8 @@
       </c>
       <c r="BX154" s="62" t="inlineStr">
         <is>
-          <t>George Baird validating</t>
-        </is>
-      </c>
-      <c r="BY154" s="63" t="n">
-        <v>46062</v>
+          <t>George Baird (v)</t>
+        </is>
       </c>
       <c r="BZ154" s="62" t="inlineStr">
         <is>
@@ -34890,11 +34849,6 @@
       <c r="CA154" s="63" t="n">
         <v>46062</v>
       </c>
-      <c r="CE154" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">George Baird validating / Alec Hickey </t>
-        </is>
-      </c>
       <c r="CG154" s="62" t="inlineStr">
         <is>
           <t>Owen</t>
@@ -34965,7 +34919,10 @@
       <c r="EH154" s="63" t="n">
         <v>46111</v>
       </c>
-      <c r="EK154" s="62" t="inlineStr">
+      <c r="GH154" s="63" t="n">
+        <v>46038</v>
+      </c>
+      <c r="GJ154" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. Self build. Delay to confirming procedure due to Insp training and late Q sub from LPA. Missed DL target due to using last cases for new Insps in training</t>
         </is>
@@ -35060,33 +35017,17 @@
       </c>
       <c r="BX155" s="62" t="inlineStr">
         <is>
-          <t>George Baird validating</t>
-        </is>
-      </c>
-      <c r="BY155" s="63" t="n">
-        <v>46080</v>
+          <t>George Baird (v)</t>
+        </is>
       </c>
       <c r="BZ155" s="62" t="inlineStr">
         <is>
-          <t>Owen Woodwards</t>
+          <t>Alec Hickey</t>
         </is>
       </c>
       <c r="CA155" s="63" t="n">
         <v>46080</v>
       </c>
-      <c r="CB155" s="62" t="inlineStr">
-        <is>
-          <t>Alec Hickey</t>
-        </is>
-      </c>
-      <c r="CC155" s="63" t="n">
-        <v>46080</v>
-      </c>
-      <c r="CE155" s="62" t="inlineStr">
-        <is>
-          <t>George Baird validating / Owen Woodwards / Alec Hickey</t>
-        </is>
-      </c>
       <c r="CG155" s="62" t="inlineStr">
         <is>
           <t>Cullum</t>
@@ -35141,7 +35082,10 @@
       <c r="EH155" s="63" t="n">
         <v>46121</v>
       </c>
-      <c r="EK155" s="62" t="inlineStr">
+      <c r="GH155" s="63" t="n">
+        <v>46049</v>
+      </c>
+      <c r="GJ155" s="62" t="inlineStr">
         <is>
           <t>BNG exemption claimed. De minimis. Missed DL target due to late information and my failure to ask for an EoT. LP</t>
         </is>

</xml_diff>